<commit_message>
Plan de test Excel : comptes et jeu de données issus de 10_jeu_de_test.sql
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fg2rtdM1t4DnuUp3bsGB2V
</commit_message>
<xml_diff>
--- a/plan_tests_site_travaux.xlsx
+++ b/plan_tests_site_travaux.xlsx
@@ -11,10 +11,11 @@
     <sheet name="Synthèse" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Cas de test" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Smoke test" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Comptes et données" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Checklists" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="Anomalies" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="Zones à risque" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Comptes de test" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Jeu de données" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Checklists" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="Anomalies" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Zones à risque" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Cas de test'!$A$1:$L$204</definedName>
@@ -29,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1950" uniqueCount="1024">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2200" uniqueCount="1175">
   <si>
     <t xml:space="preserve">Plan de test — site_travaux (ABCM Mulhouse-Lutterbach)</t>
   </si>
@@ -2683,10 +2684,22 @@
     <t xml:space="preserve">Résultat smoke (12/12 requis)</t>
   </si>
   <si>
-    <t xml:space="preserve">Comptes de test (§ 15.4.1)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Réf.</t>
+    <t xml:space="preserve">Comptes de test — source : database/sql/jeu_de_test/10_jeu_de_test.sql (domaine par défaut @recette.local)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mot de passe : choisi au chargement par charger_jeu_de_test.sh (variable MDP_RECETTE), commun à tous les comptes, jamais écrit dans le dépôt. À noter ici ou auprès du responsable de recette :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mot de passe de recette :</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(à saisir par le testeur — cellule jaune)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Réf. plan</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Id</t>
   </si>
   <si>
     <t xml:space="preserve">Login</t>
@@ -2695,169 +2708,610 @@
     <t xml:space="preserve">Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Usage</t>
+    <t xml:space="preserve">Rôle / profil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Identité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">École</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Enfants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alertes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Particularité</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cas de test concernés</t>
   </si>
   <si>
     <t xml:space="preserve">U-ADM</t>
   </si>
   <si>
-    <t xml:space="preserve">admin</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Toutes les actions d'administration</t>
+    <t xml:space="preserve">admin.recette@recette.local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Administrateur (rôle 1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[RECETTE] Administrateur</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tous droits. Compte de référence pour la configuration, le CRUD et la validation des unités.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUT-01, TRV-12, UNI-*, IMP-*, TRA-*, BOF-*, API-01</t>
   </si>
   <si>
     <t xml:space="preserve">U-SYS2</t>
   </si>
   <si>
-    <t xml:space="preserve">gestion@test.local</t>
-  </si>
-  <si>
-    <t xml:space="preserve">rôle restreint</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Vérifier le cloisonnement entre rôles sys</t>
-  </si>
-  <si>
-    <t xml:space="preserve">famille1@test.local</t>
-  </si>
-  <si>
-    <t xml:space="preserve">role_famille (2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Famille école M, 2 enfants, 0 unité</t>
+    <t xml:space="preserve">restreint.recette@recette.local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Profil restreint (rôle 9001)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[RECETTE] Profil restreint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rôle valide mais limité : droits recopiés du rôle Famille. Sert au cloisonnement entre deux profils sys.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACL-04, ACL-06, BOF-08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">famille1@recette.local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Famille (rôle 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Martin Claire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 (Lea, Tom)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WORK_REGISTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parcours nominal, 0 unité validée. Inscrite à T-FUTUR (désinscription) et à T-PASSE, T-ACTION. 2 e-mails complémentaires (conjoint, contact de secours). Second référent de session (trombi 9003).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUT-04, TRV-01 à TRV-10, FAM-01, FAM-04, CAN-*, ACL-11, MAI-01</t>
   </si>
   <si>
     <t xml:space="preserve">U-FAM2</t>
   </si>
   <si>
-    <t xml:space="preserve">famille2@test.local</t>
-  </si>
-  <si>
-    <t xml:space="preserve">role_famille</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Famille école L, unités déjà validées</t>
+    <t xml:space="preserve">famille2@recette.local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dubois Marc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 (Emma)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aucune (non abonnée)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unités déjà validées (T-VIEUX + 3 unités complémentaires). Inscrite à T-PLEIN, T-PASSE, T-ACTION, T-DERNIERE-PLACE. Candidature en attente à la commission TRAVAUX.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FAM-01, UNI-09, UNI-10, MAI-07, ORG-06, ORG-07, CAN-10</t>
   </si>
   <si>
     <t xml:space="preserve">U-REF</t>
   </si>
   <si>
-    <t xml:space="preserve">referent@test.local</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Référente de T-FUTUR et T-PASSE</t>
+    <t xml:space="preserve">referent@recette.local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Famille référente (rôle 2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Leroy Sophie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WORK_REGISTER, WORK_UNREGISTER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Référente principale (trombi 9001, classif reftra) de T-FUTUR, T-PASSE, T-ACTION, T-VIEUX… 2 unités complémentaires. Porte les 3 jetons de validation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REF-01 à REF-11, MAI-01, CRO-06, CRO-07</t>
   </si>
   <si>
     <t xml:space="preserve">U-LEGACY</t>
   </si>
   <si>
-    <t xml:space="preserve">legacy@test.local</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mot de passe encore en hash MD5/crypt() (test de migration bcrypt)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U-DELTA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">compte Delta de test</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Connexion SSO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Données métier (§ 15.4.2)</t>
+    <t xml:space="preserve">legacy@recette.local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ancien Paul</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mot de passe stocké en MD5 : doit migrer en bcrypt ($2y$) à la première connexion.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AUT-05, SEC-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U-FAM3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">famille3@recette.local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Petit Julie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B (les deux)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">aucune</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inscrite à T-PLEIN, T-PASSE, T-DERNIERE-PLACE et au créneau cantine du vendredi (saturé). Responsable de commission BUREAU (trombi RT) et membre simple TRAVAUX (ME).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CAN-05, TRV-07, TRV-11, ORG-01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U-FAM4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">famille.import@recette.local</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Import Test</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 (Import Enfant1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cible de l'import CSV : adresse « à mettre à jour », modifiée par import_ok.csv.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IMP-01 à IMP-09</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Écarts avec le § 15.4.1 de DOCUMENTATION.md</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Les logins du plan (admin, gestion@test.local, famille1@test.local…) sont remplacés par ceux du jeu de test : admin.recette@, restreint.recette@, famille1@… (domaine @recette.local, modifiable via @MAIL_DOM dans le script SQL).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• U-FAM3 (école B) et U-FAM4 (cible d'import) n'existent que dans le jeu de test ; U-DELTA (SSO) n'est pas créé par le jeu : prévoir un compte Delta réel pour AUT-06.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Tous les identifiants du jeu sont dans la plage 9000–9999 ; retrait complet avec 90_purge_jeu_de_test.sql ou POST Api/jeu_de_test {"action":"purge"} (travaux.allowTestData requis).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• ATTENTION : à n'utiliser que sur l'environnement de recette — comptes à mot de passe commun et jetons de valeur publique.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeu de données de recette — source : 10_jeu_de_test.sql (dates relatives au jour de chargement, J = jour du chargement)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sessions de travaux (table travaux)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unités</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Places</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accès école</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ce qu'elle permet de tester</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-BROUILLON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J+20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Brouillon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invisible côté famille (TRV-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-FUTUR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J+15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Publié</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inscription nominale ; U-FAM1 déjà inscrite pour tester la désinscription (TRV-05, TRV-08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-PLEIN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J+10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">B</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Session complète : U-FAM2 et U-FAM3 inscrites (TRV-07)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-PASSE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J−5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 inscrits non validés (U-FAM1, U-FAM2 couple, U-FAM3) : validation référent (REF-02)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-VIEUX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J−45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GOU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Archivage automatique &gt; 30 jours (TRV-15) ; déjà validée pour U-FAM2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-URG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(aucune)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">URG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sans date, jamais archivée (TRV-15, TRV-19)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-LUT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J+12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Invisible pour une famille de Mulhouse (TRV-03)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-AN-1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J−300</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Année civile précédente (TRV-04)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-ACTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J−3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DEC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Type Action dans la file de validation (UNI-01) ; 2 inscrits non validés</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-REF-KO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J+6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Référent à chaîne rompue : aucun mail, aucune erreur (CRO-08, MAI-06, ORG-08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-DERNIERE-PLACE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J+8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 places prises sur 3 ; second référent (Martin Claire) : concurrence (TRV-11, PER-04)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-CAN lundi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lundi de la semaine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">can</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantine 11h45–13h30 (CAN-03, CAN-04)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-CAN mardi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mardi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantine</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-CAN jeudi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">jeudi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantine (le mercredi est volontairement absent)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-CAN vendredi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vendredi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Créneau saturé : U-FAM3 inscrite (CAN-05)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jetons de validation référent (validation_tokens) — URL : &lt;base_url&gt;/Admwork_controller/validate_by_token/&lt;jeton&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Comportement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Session</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Famille réf.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expiration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jeton (valeur fixe, 64 caractères hexadécimaux)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VALIDE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9004 (T-PASSE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9003 (U-REF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J+25</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a1b2c3d4e5f60718293a4b5c6d7e8f90a1b2c3d4e5f60718293a4b5c6d7e8f90  → REF-04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EXPIRÉ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9009 (T-ACTION)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J−1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b1b2c3d4e5f60718293a4b5c6d7e8f90a1b2c3d4e5f60718293a4b5c6d7e8f91  → REF-06 : refus attendu</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DÉJÀ UTILISÉ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9005 (T-VIEUX)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J+10 (used_at = J−2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">c1b2c3d4e5f60718293a4b5c6d7e8f90a1b2c3d4e5f60718293a4b5c6d7e8f92  → REF-07 : refus, pas de double comptage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Inscriptions (table infos)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Famille</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Participants</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unités prévues</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unités validées</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-PLEIN 9003</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mr</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mme</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-PASSE 9004</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Both</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-ACTION 9009</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-DERNIERE-PLACE 9011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-VIEUX 9005</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-FUTUR 9002</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T-CAN vendredi 9024</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unités complémentaires hors session (table unites)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Motif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J−20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Don de matériel : 3 unités accordées hors session</t>
+  </si>
+  <si>
+    <t xml:space="preserve">J−15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Animation de session : 2 unités accordées</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total d'unités validées attendu par famille (contrôle FAM-01 / UNI-10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sessions validées</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unités hors session</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 unité (T-VIEUX) + 3 unités complémentaires</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commissions et référents (groupes / groupes_member / trombi)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trombi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Id commission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Classif.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Référent proposé sur les sessions ?</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAVAUX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reftra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9003 Leroy Sophie (U-REF)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oui — référente principale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_fam non numérique (Chaîne Rompue)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oui, mais aucune famille derrière (ORG-08, CRO-08)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9001 Martin Claire (U-FAM1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oui — second référent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BUREAU</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9005 Petit Julie (U-FAM3)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Oui — responsable de commission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non — membre simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Autres données</t>
   </si>
   <si>
     <t xml:space="preserve">Objet</t>
   </si>
   <si>
-    <t xml:space="preserve">Caractéristiques</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-BROUILLON</t>
-  </si>
-  <si>
-    <t xml:space="preserve">travaux</t>
-  </si>
-  <si>
-    <t xml:space="preserve">statut=0, date future — ne doit pas apparaître côté famille</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-FUTUR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type=TRA, statut=1, date J+15, nb_inscrits_max=4, nb_units=2, accespar=M, référent = U-REF</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-PLEIN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nb_inscrits_max=2 et déjà 2 inscrits — test de saturation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-PASSE</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date J-5, non archivé — validation référent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-VIEUX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">date J-45, archived=0 — test d'archivage automatique</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-URG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type=URG, sans date — ne doit jamais être archivé</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-LUT</t>
-  </si>
-  <si>
-    <t xml:space="preserve">accespar=L — invisible pour U-FAM1 (école M)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-AN-1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">civil_year=2024-2025 — cloisonnement par année</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T-CAN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">type=can, généré par le module cantine</t>
-  </si>
-  <si>
-    <t xml:space="preserve">G-COM</t>
-  </si>
-  <si>
-    <t xml:space="preserve">groupes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commission type=com avec 2 membres et 1 candidature en attente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CSV-OK</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fichier</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Export ABCM valide, 10 familles dont 2 nouvelles et 1 modifiée</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CSV-KO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Même fichier avec colonnes manquantes / encodage erroné</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jeu de données SQL de recette : database/sql/jeu_de_test/ (ne jamais charger en production).</t>
+    <t xml:space="preserve">Détail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">U-FAM2 (Dubois Marc) → commission TRAVAUX 9001, en attente : à accepter puis refuser (ORG-06, ORG-07)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cantine config</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lundi, mardi, jeudi actifs (4 créneaux), vendredi 1 créneau, mercredi inactif — école M, 1 unité, 11h45–13h30, référent trombi 9001</t>
+  </si>
+  <si>
+    <t xml:space="preserve">File sendmail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECETTE-01 → famille1@, statut 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECETTE-02 → famille2@, statut 0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RECETTE-03 → referent@, statut 0 (CRO-01 / CRO-03 : 3 mails en attente)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichiers CSV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">database/sql/jeu_de_test/csv/import_ok.csv (CSV-OK) et import_ko.csv (CSV-KO)</t>
   </si>
   <si>
     <t xml:space="preserve">Rubrique</t>
@@ -3113,7 +3567,7 @@
     <numFmt numFmtId="166" formatCode="0"/>
     <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -3178,8 +3632,15 @@
       <family val="0"/>
       <charset val="1"/>
     </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3190,6 +3651,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E78"/>
         <bgColor rgb="FF003366"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF99"/>
+        <bgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -3242,7 +3709,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="16">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3293,6 +3760,18 @@
     </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -3385,7 +3864,7 @@
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
-      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFFFEB9C"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
@@ -3402,7 +3881,7 @@
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFC6EFCE"/>
-      <rgbColor rgb="FFFFEB9C"/>
+      <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -10924,309 +11403,378 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:K19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="50"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="7"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="24"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="40"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="13" t="s">
         <v>884</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="14" t="s">
         <v>885</v>
       </c>
-      <c r="B2" s="3" t="s">
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
         <v>886</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C3" s="15"/>
+      <c r="D3" s="2" t="s">
         <v>887</v>
       </c>
-      <c r="D2" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="E2" s="3" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>888</v>
       </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="s">
+      <c r="B5" s="3" t="s">
         <v>889</v>
       </c>
-      <c r="B3" s="10" t="s">
+      <c r="C5" s="3" t="s">
         <v>890</v>
       </c>
-      <c r="C3" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D3" s="10" t="s">
-        <v>890</v>
-      </c>
-      <c r="E3" s="10" t="s">
+      <c r="D5" s="3" t="s">
         <v>891</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="E5" s="3" t="s">
         <v>892</v>
       </c>
-      <c r="B4" s="10" t="s">
+      <c r="F5" s="3" t="s">
         <v>893</v>
       </c>
-      <c r="C4" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D4" s="10" t="s">
+      <c r="G5" s="3" t="s">
         <v>894</v>
       </c>
-      <c r="E4" s="10" t="s">
+      <c r="H5" s="3" t="s">
         <v>895</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="10" t="s">
+      <c r="I5" s="3" t="s">
         <v>896</v>
       </c>
-      <c r="C5" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="D5" s="10" t="s">
+      <c r="J5" s="3" t="s">
         <v>897</v>
       </c>
-      <c r="E5" s="10" t="s">
+      <c r="K5" s="3" t="s">
         <v>898</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
         <v>899</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C6" s="10" t="s">
         <v>900</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="D6" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E6" s="10" t="s">
+        <v>901</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>902</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J6" s="10" t="s">
+        <v>903</v>
+      </c>
+      <c r="K6" s="10" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>905</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>906</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="E7" s="10" t="s">
+        <v>907</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>908</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J7" s="10" t="s">
+        <v>909</v>
+      </c>
+      <c r="K7" s="10" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>911</v>
+      </c>
+      <c r="D8" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="10" t="s">
-        <v>901</v>
-      </c>
-      <c r="E6" s="10" t="s">
-        <v>902</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="s">
-        <v>903</v>
-      </c>
-      <c r="B7" s="10" t="s">
-        <v>904</v>
-      </c>
-      <c r="C7" s="10" t="s">
+      <c r="E8" s="10" t="s">
+        <v>912</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>913</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>915</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>916</v>
+      </c>
+      <c r="J8" s="10" t="s">
+        <v>917</v>
+      </c>
+      <c r="K8" s="10" t="s">
+        <v>918</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>919</v>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>920</v>
+      </c>
+      <c r="D9" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="D7" s="10" t="s">
-        <v>901</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>905</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="s">
-        <v>906</v>
-      </c>
-      <c r="B8" s="10" t="s">
-        <v>907</v>
-      </c>
-      <c r="C8" s="10" t="s">
+      <c r="E9" s="10" t="s">
+        <v>912</v>
+      </c>
+      <c r="F9" s="10" t="s">
+        <v>921</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>922</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>923</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>924</v>
+      </c>
+      <c r="J9" s="10" t="s">
+        <v>925</v>
+      </c>
+      <c r="K9" s="10" t="s">
+        <v>926</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>927</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>9003</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>928</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="D8" s="10" t="s">
-        <v>901</v>
-      </c>
-      <c r="E8" s="10" t="s">
-        <v>908</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="s">
-        <v>909</v>
-      </c>
-      <c r="B9" s="10" t="s">
-        <v>910</v>
-      </c>
-      <c r="C9" s="10" t="s">
+      <c r="E10" s="10" t="s">
+        <v>929</v>
+      </c>
+      <c r="F10" s="10" t="s">
+        <v>930</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>850</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>931</v>
+      </c>
+      <c r="J10" s="10" t="s">
+        <v>932</v>
+      </c>
+      <c r="K10" s="10" t="s">
+        <v>933</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>934</v>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>9004</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>935</v>
+      </c>
+      <c r="D11" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="D9" s="10" t="s">
+      <c r="E11" s="10" t="s">
+        <v>912</v>
+      </c>
+      <c r="F11" s="10" t="s">
+        <v>936</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H11" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="E9" s="10" t="s">
-        <v>911</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="s">
+      <c r="I11" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J11" s="10" t="s">
+        <v>937</v>
+      </c>
+      <c r="K11" s="10" t="s">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>939</v>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>9005</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>940</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="10" t="s">
         <v>912</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
-        <v>885</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>913</v>
-      </c>
-      <c r="C13" s="3" t="s">
+      <c r="F12" s="10" t="s">
+        <v>941</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>942</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>853</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>943</v>
+      </c>
+      <c r="J12" s="10" t="s">
+        <v>944</v>
+      </c>
+      <c r="K12" s="10" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>946</v>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>9006</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>947</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>66</v>
+      </c>
+      <c r="E13" s="10" t="s">
+        <v>912</v>
+      </c>
+      <c r="F13" s="10" t="s">
+        <v>948</v>
+      </c>
+      <c r="G13" s="10" t="s">
         <v>914</v>
       </c>
-    </row>
-    <row r="14" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="s">
-        <v>915</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>917</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="102.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
-        <v>918</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>919</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>920</v>
-      </c>
-      <c r="B16" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>921</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
-        <v>922</v>
-      </c>
-      <c r="B17" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C17" s="10" t="s">
-        <v>923</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="s">
-        <v>924</v>
-      </c>
-      <c r="B18" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>925</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
-        <v>926</v>
-      </c>
-      <c r="B19" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C19" s="10" t="s">
-        <v>927</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="s">
-        <v>928</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>929</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="s">
-        <v>930</v>
-      </c>
-      <c r="B21" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C21" s="10" t="s">
-        <v>931</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="s">
-        <v>932</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>916</v>
-      </c>
-      <c r="C22" s="10" t="s">
-        <v>933</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="s">
-        <v>934</v>
-      </c>
-      <c r="B23" s="10" t="s">
-        <v>935</v>
-      </c>
-      <c r="C23" s="10" t="s">
-        <v>936</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="s">
-        <v>937</v>
-      </c>
-      <c r="B24" s="10" t="s">
-        <v>938</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>939</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="s">
-        <v>940</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>938</v>
-      </c>
-      <c r="C25" s="10" t="s">
-        <v>941</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2" t="s">
-        <v>942</v>
+      <c r="H13" s="10" t="s">
+        <v>949</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="J13" s="10" t="s">
+        <v>950</v>
+      </c>
+      <c r="K13" s="10" t="s">
+        <v>951</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="8" t="s">
+        <v>952</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="14" t="s">
+        <v>953</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="14" t="s">
+        <v>955</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="14" t="s">
+        <v>956</v>
       </c>
     </row>
   </sheetData>
@@ -11245,6 +11793,1356 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
+  <dimension ref="A1:I68"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="60"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
+        <v>957</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="8" t="s">
+        <v>958</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>888</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>891</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>959</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>960</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>961</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>962</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="10" t="s">
+        <v>963</v>
+      </c>
+      <c r="B5" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C5" s="10" t="s">
+        <v>964</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F5" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>966</v>
+      </c>
+      <c r="I5" s="10" t="s">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>968</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>969</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F6" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H6" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I6" s="10" t="s">
+        <v>971</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="10" t="s">
+        <v>972</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>9003</v>
+      </c>
+      <c r="C7" s="10" t="s">
+        <v>973</v>
+      </c>
+      <c r="D7" s="10" t="s">
+        <v>974</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G7" s="10" t="s">
+        <v>975</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I7" s="10" t="s">
+        <v>976</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="10" t="s">
+        <v>977</v>
+      </c>
+      <c r="B8" s="10" t="n">
+        <v>9004</v>
+      </c>
+      <c r="C8" s="10" t="s">
+        <v>978</v>
+      </c>
+      <c r="D8" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="E8" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F8" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>979</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="10" t="s">
+        <v>980</v>
+      </c>
+      <c r="B9" s="10" t="n">
+        <v>9005</v>
+      </c>
+      <c r="C9" s="10" t="s">
+        <v>981</v>
+      </c>
+      <c r="D9" s="10" t="s">
+        <v>982</v>
+      </c>
+      <c r="E9" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="G9" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H9" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I9" s="10" t="s">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="10" t="s">
+        <v>984</v>
+      </c>
+      <c r="B10" s="10" t="n">
+        <v>9006</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>985</v>
+      </c>
+      <c r="D10" s="10" t="s">
+        <v>986</v>
+      </c>
+      <c r="E10" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="G10" s="10" t="s">
+        <v>975</v>
+      </c>
+      <c r="H10" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I10" s="10" t="s">
+        <v>987</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="10" t="s">
+        <v>988</v>
+      </c>
+      <c r="B11" s="10" t="n">
+        <v>9007</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>989</v>
+      </c>
+      <c r="D11" s="10" t="s">
+        <v>990</v>
+      </c>
+      <c r="E11" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F11" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G11" s="10" t="s">
+        <v>922</v>
+      </c>
+      <c r="H11" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I11" s="10" t="s">
+        <v>991</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="10" t="s">
+        <v>992</v>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>9008</v>
+      </c>
+      <c r="C12" s="10" t="s">
+        <v>993</v>
+      </c>
+      <c r="D12" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="E12" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G12" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H12" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I12" s="10" t="s">
+        <v>994</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="10" t="s">
+        <v>995</v>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>9009</v>
+      </c>
+      <c r="C13" s="10" t="s">
+        <v>996</v>
+      </c>
+      <c r="D13" s="10" t="s">
+        <v>997</v>
+      </c>
+      <c r="E13" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H13" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I13" s="10" t="s">
+        <v>998</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>999</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>9010</v>
+      </c>
+      <c r="C14" s="10" t="s">
+        <v>1000</v>
+      </c>
+      <c r="D14" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="E14" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F14" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I14" s="10" t="s">
+        <v>1001</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="10" t="s">
+        <v>1002</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>9011</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>1003</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>965</v>
+      </c>
+      <c r="E15" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G15" s="10" t="s">
+        <v>975</v>
+      </c>
+      <c r="H15" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I15" s="10" t="s">
+        <v>1004</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="10" t="s">
+        <v>1005</v>
+      </c>
+      <c r="B16" s="10" t="n">
+        <v>9020</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>1006</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E16" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H16" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I16" s="10" t="s">
+        <v>1008</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="10" t="s">
+        <v>1009</v>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>9021</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>1010</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E17" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H17" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I17" s="10" t="s">
+        <v>1011</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="s">
+        <v>1012</v>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>9023</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>1013</v>
+      </c>
+      <c r="D18" s="10" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E18" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G18" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H18" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I18" s="10" t="s">
+        <v>1014</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
+        <v>1015</v>
+      </c>
+      <c r="B19" s="10" t="n">
+        <v>9024</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>1016</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>1007</v>
+      </c>
+      <c r="E19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>914</v>
+      </c>
+      <c r="H19" s="10" t="s">
+        <v>970</v>
+      </c>
+      <c r="I19" s="10" t="s">
+        <v>1017</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="8" t="s">
+        <v>1018</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>1019</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>1021</v>
+      </c>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3" t="s">
+        <v>1022</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>1023</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="10" t="s">
+        <v>1024</v>
+      </c>
+      <c r="B23" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>1025</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>1026</v>
+      </c>
+      <c r="E23" s="10"/>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="10" t="s">
+        <v>1027</v>
+      </c>
+      <c r="I23" s="10" t="s">
+        <v>1028</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="10" t="s">
+        <v>1029</v>
+      </c>
+      <c r="B24" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C24" s="10" t="s">
+        <v>1030</v>
+      </c>
+      <c r="D24" s="10" t="s">
+        <v>1026</v>
+      </c>
+      <c r="E24" s="10"/>
+      <c r="F24" s="10"/>
+      <c r="G24" s="10"/>
+      <c r="H24" s="10" t="s">
+        <v>1031</v>
+      </c>
+      <c r="I24" s="10" t="s">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="10" t="s">
+        <v>1033</v>
+      </c>
+      <c r="B25" s="10" t="n">
+        <v>9003</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>1034</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>1026</v>
+      </c>
+      <c r="E25" s="10"/>
+      <c r="F25" s="10"/>
+      <c r="G25" s="10"/>
+      <c r="H25" s="10" t="s">
+        <v>1035</v>
+      </c>
+      <c r="I25" s="10" t="s">
+        <v>1036</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="8" t="s">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>1020</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>1039</v>
+      </c>
+      <c r="E28" s="3" t="s">
+        <v>891</v>
+      </c>
+      <c r="F28" s="3" t="s">
+        <v>1040</v>
+      </c>
+      <c r="G28" s="3" t="s">
+        <v>1041</v>
+      </c>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="10" t="s">
+        <v>919</v>
+      </c>
+      <c r="B29" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C29" s="10" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D29" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>1043</v>
+      </c>
+      <c r="F29" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="10" t="s">
+        <v>939</v>
+      </c>
+      <c r="B30" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>1042</v>
+      </c>
+      <c r="D30" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="10" t="s">
+        <v>1044</v>
+      </c>
+      <c r="F30" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G30" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B31" s="10" t="n">
+        <v>9003</v>
+      </c>
+      <c r="C31" s="10" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D31" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="10" t="s">
+        <v>1043</v>
+      </c>
+      <c r="F31" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G31" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="10" t="s">
+        <v>919</v>
+      </c>
+      <c r="B32" s="10" t="n">
+        <v>9004</v>
+      </c>
+      <c r="C32" s="10" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D32" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E32" s="10" t="s">
+        <v>1046</v>
+      </c>
+      <c r="F32" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="G32" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="10"/>
+      <c r="I32" s="10"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="s">
+        <v>939</v>
+      </c>
+      <c r="B33" s="10" t="n">
+        <v>9005</v>
+      </c>
+      <c r="C33" s="10" t="s">
+        <v>1045</v>
+      </c>
+      <c r="D33" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="10" t="s">
+        <v>1044</v>
+      </c>
+      <c r="F33" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G33" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="10"/>
+      <c r="I33" s="10"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B34" s="10" t="n">
+        <v>9006</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D34" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="10" t="s">
+        <v>1043</v>
+      </c>
+      <c r="F34" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="G34" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="10"/>
+      <c r="I34" s="10"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="s">
+        <v>919</v>
+      </c>
+      <c r="B35" s="10" t="n">
+        <v>9007</v>
+      </c>
+      <c r="C35" s="10" t="s">
+        <v>1047</v>
+      </c>
+      <c r="D35" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E35" s="10" t="s">
+        <v>1046</v>
+      </c>
+      <c r="F35" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="G35" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="10"/>
+      <c r="I35" s="10"/>
+    </row>
+    <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="10" t="s">
+        <v>919</v>
+      </c>
+      <c r="B36" s="10" t="n">
+        <v>9008</v>
+      </c>
+      <c r="C36" s="10" t="s">
+        <v>1048</v>
+      </c>
+      <c r="D36" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E36" s="10" t="s">
+        <v>1043</v>
+      </c>
+      <c r="F36" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G36" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="10"/>
+      <c r="I36" s="10"/>
+    </row>
+    <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="s">
+        <v>939</v>
+      </c>
+      <c r="B37" s="10" t="n">
+        <v>9009</v>
+      </c>
+      <c r="C37" s="10" t="s">
+        <v>1048</v>
+      </c>
+      <c r="D37" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="10" t="s">
+        <v>1044</v>
+      </c>
+      <c r="F37" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G37" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="10"/>
+      <c r="I37" s="10"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="10" t="s">
+        <v>919</v>
+      </c>
+      <c r="B38" s="10" t="n">
+        <v>9010</v>
+      </c>
+      <c r="C38" s="10" t="s">
+        <v>1049</v>
+      </c>
+      <c r="D38" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="10" t="s">
+        <v>1043</v>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H38" s="10"/>
+      <c r="I38" s="10"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B39" s="10" t="n">
+        <v>9011</v>
+      </c>
+      <c r="C39" s="10" t="s">
+        <v>1050</v>
+      </c>
+      <c r="D39" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E39" s="10" t="s">
+        <v>1043</v>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="G39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="10"/>
+      <c r="I39" s="10"/>
+    </row>
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10" t="s">
+        <v>939</v>
+      </c>
+      <c r="B40" s="10" t="n">
+        <v>9012</v>
+      </c>
+      <c r="C40" s="10" t="s">
+        <v>1051</v>
+      </c>
+      <c r="D40" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="E40" s="10" t="s">
+        <v>1044</v>
+      </c>
+      <c r="F40" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="10"/>
+      <c r="I40" s="10"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="8" t="s">
+        <v>1052</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="3" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B43" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>959</v>
+      </c>
+      <c r="E43" s="3"/>
+      <c r="F43" s="3"/>
+      <c r="G43" s="3"/>
+      <c r="H43" s="3"/>
+      <c r="I43" s="3" t="s">
+        <v>1053</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="10" t="s">
+        <v>919</v>
+      </c>
+      <c r="B44" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C44" s="10" t="s">
+        <v>1054</v>
+      </c>
+      <c r="D44" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E44" s="10"/>
+      <c r="F44" s="10"/>
+      <c r="G44" s="10"/>
+      <c r="H44" s="10"/>
+      <c r="I44" s="10" t="s">
+        <v>1055</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="10" t="s">
+        <v>927</v>
+      </c>
+      <c r="B45" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C45" s="10" t="s">
+        <v>1056</v>
+      </c>
+      <c r="D45" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E45" s="10"/>
+      <c r="F45" s="10"/>
+      <c r="G45" s="10"/>
+      <c r="H45" s="10"/>
+      <c r="I45" s="10" t="s">
+        <v>1057</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="8" t="s">
+        <v>1058</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>1038</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3" t="s">
+        <v>1059</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>1060</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="F48" s="3"/>
+      <c r="G48" s="3"/>
+      <c r="H48" s="3"/>
+      <c r="I48" s="3"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B49" s="10"/>
+      <c r="C49" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D49" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" s="10" t="n">
+        <f aca="false">C49+D49</f>
+        <v>0</v>
+      </c>
+      <c r="F49" s="10"/>
+      <c r="G49" s="10"/>
+      <c r="H49" s="10"/>
+      <c r="I49" s="10"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10" t="s">
+        <v>919</v>
+      </c>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="D50" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E50" s="10" t="n">
+        <f aca="false">C50+D50</f>
+        <v>4</v>
+      </c>
+      <c r="F50" s="10"/>
+      <c r="G50" s="10"/>
+      <c r="H50" s="10"/>
+      <c r="I50" s="10" t="s">
+        <v>1061</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="10" t="s">
+        <v>927</v>
+      </c>
+      <c r="B51" s="10"/>
+      <c r="C51" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D51" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="E51" s="10" t="n">
+        <f aca="false">C51+D51</f>
+        <v>2</v>
+      </c>
+      <c r="F51" s="10"/>
+      <c r="G51" s="10"/>
+      <c r="H51" s="10"/>
+      <c r="I51" s="10"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="8" t="s">
+        <v>1062</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="3" t="s">
+        <v>1063</v>
+      </c>
+      <c r="B54" s="3" t="s">
+        <v>1064</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>1065</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>1066</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>1038</v>
+      </c>
+      <c r="F54" s="3"/>
+      <c r="G54" s="3"/>
+      <c r="H54" s="3"/>
+      <c r="I54" s="3" t="s">
+        <v>1067</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="B55" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C55" s="10" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>1070</v>
+      </c>
+      <c r="F55" s="10"/>
+      <c r="G55" s="10"/>
+      <c r="H55" s="10"/>
+      <c r="I55" s="10" t="s">
+        <v>1071</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="B56" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C56" s="10" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E56" s="10" t="s">
+        <v>1072</v>
+      </c>
+      <c r="F56" s="10"/>
+      <c r="G56" s="10"/>
+      <c r="H56" s="10"/>
+      <c r="I56" s="10" t="s">
+        <v>1073</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="10" t="n">
+        <v>9003</v>
+      </c>
+      <c r="B57" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C57" s="10" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>1069</v>
+      </c>
+      <c r="E57" s="10" t="s">
+        <v>1074</v>
+      </c>
+      <c r="F57" s="10"/>
+      <c r="G57" s="10"/>
+      <c r="H57" s="10"/>
+      <c r="I57" s="10" t="s">
+        <v>1075</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="10" t="n">
+        <v>9004</v>
+      </c>
+      <c r="B58" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C58" s="10" t="s">
+        <v>1076</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>1077</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F58" s="10"/>
+      <c r="G58" s="10"/>
+      <c r="H58" s="10"/>
+      <c r="I58" s="10" t="s">
+        <v>1079</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="10" t="n">
+        <v>9005</v>
+      </c>
+      <c r="B59" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C59" s="10" t="s">
+        <v>1068</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>1080</v>
+      </c>
+      <c r="E59" s="10" t="s">
+        <v>1078</v>
+      </c>
+      <c r="F59" s="10"/>
+      <c r="G59" s="10"/>
+      <c r="H59" s="10"/>
+      <c r="I59" s="10" t="s">
+        <v>1081</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="8" t="s">
+        <v>1082</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="3" t="s">
+        <v>1083</v>
+      </c>
+      <c r="B62" s="3" t="s">
+        <v>889</v>
+      </c>
+      <c r="C62" s="3" t="s">
+        <v>1084</v>
+      </c>
+      <c r="D62" s="3"/>
+      <c r="E62" s="3"/>
+      <c r="F62" s="3"/>
+      <c r="G62" s="3"/>
+      <c r="H62" s="3"/>
+      <c r="I62" s="3"/>
+    </row>
+    <row r="63" customFormat="false" ht="91" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="10" t="s">
+        <v>474</v>
+      </c>
+      <c r="B63" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C63" s="10" t="s">
+        <v>1085</v>
+      </c>
+      <c r="D63" s="10"/>
+      <c r="E63" s="10"/>
+      <c r="F63" s="10"/>
+      <c r="G63" s="10"/>
+      <c r="H63" s="10"/>
+      <c r="I63" s="10"/>
+    </row>
+    <row r="64" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="10" t="s">
+        <v>1086</v>
+      </c>
+      <c r="B64" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C64" s="10" t="s">
+        <v>1087</v>
+      </c>
+      <c r="D64" s="10"/>
+      <c r="E64" s="10"/>
+      <c r="F64" s="10"/>
+      <c r="G64" s="10"/>
+      <c r="H64" s="10"/>
+      <c r="I64" s="10"/>
+    </row>
+    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="10" t="s">
+        <v>1088</v>
+      </c>
+      <c r="B65" s="10" t="n">
+        <v>9001</v>
+      </c>
+      <c r="C65" s="10" t="s">
+        <v>1089</v>
+      </c>
+      <c r="D65" s="10"/>
+      <c r="E65" s="10"/>
+      <c r="F65" s="10"/>
+      <c r="G65" s="10"/>
+      <c r="H65" s="10"/>
+      <c r="I65" s="10"/>
+    </row>
+    <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="10" t="s">
+        <v>1088</v>
+      </c>
+      <c r="B66" s="10" t="n">
+        <v>9002</v>
+      </c>
+      <c r="C66" s="10" t="s">
+        <v>1090</v>
+      </c>
+      <c r="D66" s="10"/>
+      <c r="E66" s="10"/>
+      <c r="F66" s="10"/>
+      <c r="G66" s="10"/>
+      <c r="H66" s="10"/>
+      <c r="I66" s="10"/>
+    </row>
+    <row r="67" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="10" t="s">
+        <v>1088</v>
+      </c>
+      <c r="B67" s="10" t="n">
+        <v>9003</v>
+      </c>
+      <c r="C67" s="10" t="s">
+        <v>1091</v>
+      </c>
+      <c r="D67" s="10"/>
+      <c r="E67" s="10"/>
+      <c r="F67" s="10"/>
+      <c r="G67" s="10"/>
+      <c r="H67" s="10"/>
+      <c r="I67" s="10"/>
+    </row>
+    <row r="68" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="10" t="s">
+        <v>1092</v>
+      </c>
+      <c r="B68" s="10" t="s">
+        <v>57</v>
+      </c>
+      <c r="C68" s="10" t="s">
+        <v>1093</v>
+      </c>
+      <c r="D68" s="10"/>
+      <c r="E68" s="10"/>
+      <c r="F68" s="10"/>
+      <c r="G68" s="10"/>
+      <c r="H68" s="10"/>
+      <c r="I68" s="10"/>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:D34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
@@ -11256,13 +13154,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>943</v>
+        <v>1094</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>944</v>
+        <v>1095</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>945</v>
+        <v>1096</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>49</v>
@@ -11270,397 +13168,397 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>946</v>
+        <v>1097</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>947</v>
+        <v>1098</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>946</v>
+        <v>1097</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>949</v>
+        <v>1100</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>946</v>
+        <v>1097</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>950</v>
+        <v>1101</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>946</v>
+        <v>1097</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>951</v>
+        <v>1102</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>946</v>
+        <v>1097</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>952</v>
+        <v>1103</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>946</v>
+        <v>1097</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>953</v>
+        <v>1104</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>946</v>
+        <v>1097</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>954</v>
+        <v>1105</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>946</v>
+        <v>1097</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>955</v>
+        <v>1106</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>957</v>
+        <v>1108</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>958</v>
+        <v>1109</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>959</v>
+        <v>1110</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>960</v>
+        <v>1111</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>961</v>
+        <v>1112</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>962</v>
+        <v>1113</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>963</v>
+        <v>1114</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>964</v>
+        <v>1115</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>965</v>
+        <v>1116</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>966</v>
+        <v>1117</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>967</v>
+        <v>1118</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>968</v>
+        <v>1119</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>969</v>
+        <v>1120</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>970</v>
+        <v>1121</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>971</v>
+        <v>1122</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>956</v>
+        <v>1107</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>972</v>
+        <v>1123</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>973</v>
+        <v>1124</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>974</v>
+        <v>1125</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>973</v>
+        <v>1124</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>975</v>
+        <v>1126</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>973</v>
+        <v>1124</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>976</v>
+        <v>1127</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>973</v>
+        <v>1124</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>977</v>
+        <v>1128</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>978</v>
+        <v>1129</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>979</v>
+        <v>1130</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>978</v>
+        <v>1129</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>980</v>
+        <v>1131</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>978</v>
+        <v>1129</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>981</v>
+        <v>1132</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>978</v>
+        <v>1129</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>982</v>
+        <v>1133</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>978</v>
+        <v>1129</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>983</v>
+        <v>1134</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>948</v>
+        <v>1099</v>
       </c>
       <c r="D34" s="11"/>
     </row>
@@ -11681,7 +13579,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -11707,25 +13605,25 @@
         <v>39</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>984</v>
+        <v>1135</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>985</v>
+        <v>1136</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>986</v>
+        <v>1137</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>987</v>
+        <v>1138</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>988</v>
+        <v>1139</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>989</v>
+        <v>1140</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>990</v>
+        <v>1141</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>44</v>
@@ -11734,7 +13632,7 @@
         <v>47</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>991</v>
+        <v>1142</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>46</v>
@@ -11742,34 +13640,34 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>992</v>
+        <v>1143</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>181</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>993</v>
+        <v>1144</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>994</v>
+        <v>1145</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>68</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>995</v>
+        <v>1146</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>996</v>
+        <v>1147</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>997</v>
+        <v>1148</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>997</v>
+        <v>1148</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>998</v>
+        <v>1149</v>
       </c>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
@@ -12574,7 +14472,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>999</v>
+        <v>1150</v>
       </c>
     </row>
   </sheetData>
@@ -12598,7 +14496,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
@@ -12613,21 +14511,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>1000</v>
+        <v>1151</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1001</v>
+        <v>1152</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1002</v>
+        <v>1153</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>1003</v>
+        <v>1154</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>1004</v>
+        <v>1155</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>169</v>
@@ -12635,65 +14533,65 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>1005</v>
+        <v>1156</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>1006</v>
+        <v>1157</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>1007</v>
+        <v>1158</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>1008</v>
+        <v>1159</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1009</v>
+        <v>1160</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>1010</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>1011</v>
+        <v>1162</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>1012</v>
+        <v>1163</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>1013</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>1014</v>
+        <v>1165</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1015</v>
+        <v>1166</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>1016</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>1017</v>
+        <v>1168</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>1018</v>
+        <v>1169</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>1019</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>1020</v>
+        <v>1171</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>1021</v>
+        <v>1172</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>450</v>
@@ -12701,10 +14599,10 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1022</v>
+        <v>1173</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>1023</v>
+        <v>1174</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>679</v>

</xml_diff>

<commit_message>
Plan de test Excel : statut du smoke test déduit de l'onglet Cas de test
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fg2rtdM1t4DnuUp3bsGB2V
</commit_message>
<xml_diff>
--- a/plan_tests_site_travaux.xlsx
+++ b/plan_tests_site_travaux.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2200" uniqueCount="1175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2190" uniqueCount="1178">
   <si>
     <t xml:space="preserve">Plan de test — site_travaux (ABCM Mulhouse-Lutterbach)</t>
   </si>
@@ -2573,6 +2573,9 @@
     <t xml:space="preserve">Attendu</t>
   </si>
   <si>
+    <t xml:space="preserve">Statut (déduit de « Cas de test »)</t>
+  </si>
+  <si>
     <t xml:space="preserve">1</t>
   </si>
   <si>
@@ -2681,7 +2684,13 @@
     <t xml:space="preserve">Session détruite, retour au formulaire de connexion</t>
   </si>
   <si>
-    <t xml:space="preserve">Résultat smoke (12/12 requis)</t>
+    <t xml:space="preserve">OK / total (12/12 requis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Verdict</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les colonnes Testeur, Date et Statut sont déduites de l'onglet « Cas de test » : renseigner le statut là-bas.</t>
   </si>
   <si>
     <t xml:space="preserve">Comptes de test — source : database/sql/jeu_de_test/10_jeu_de_test.sql (domaine par défaut @recette.local)</t>
@@ -3709,7 +3718,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -3759,6 +3768,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="167" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -11134,18 +11147,19 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="56"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="36"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
         <v>845</v>
       </c>
@@ -11162,7 +11176,7 @@
         <v>46</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>47</v>
+        <v>847</v>
       </c>
       <c r="G1" s="3" t="s">
         <v>49</v>
@@ -11170,224 +11184,330 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>847</v>
+        <v>848</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>848</v>
+        <v>849</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>849</v>
-      </c>
-      <c r="D2" s="11"/>
-      <c r="E2" s="12"/>
-      <c r="F2" s="11" t="s">
-        <v>5</v>
+        <v>850</v>
+      </c>
+      <c r="D2" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B2,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E2" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B2,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B2,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F2" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B2,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>851</v>
+        <v>852</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>852</v>
-      </c>
-      <c r="D3" s="11"/>
-      <c r="E3" s="12"/>
-      <c r="F3" s="11" t="s">
-        <v>5</v>
+        <v>853</v>
+      </c>
+      <c r="D3" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B3,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E3" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B3,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B3,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F3" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B3,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>854</v>
+        <v>855</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>855</v>
-      </c>
-      <c r="D4" s="11"/>
-      <c r="E4" s="12"/>
-      <c r="F4" s="11" t="s">
-        <v>5</v>
+        <v>856</v>
+      </c>
+      <c r="D4" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B4,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E4" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B4,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B4,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F4" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B4,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>856</v>
+        <v>857</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>857</v>
+        <v>858</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>858</v>
-      </c>
-      <c r="D5" s="11"/>
-      <c r="E5" s="12"/>
-      <c r="F5" s="11" t="s">
-        <v>5</v>
+        <v>859</v>
+      </c>
+      <c r="D5" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B5,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E5" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B5,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B5,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F5" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B5,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>859</v>
+        <v>860</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>860</v>
+        <v>861</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>861</v>
-      </c>
-      <c r="D6" s="11"/>
-      <c r="E6" s="12"/>
-      <c r="F6" s="11" t="s">
-        <v>5</v>
+        <v>862</v>
+      </c>
+      <c r="D6" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B6,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E6" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B6,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B6,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F6" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B6,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>862</v>
+        <v>863</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>863</v>
+        <v>864</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>864</v>
-      </c>
-      <c r="D7" s="11"/>
-      <c r="E7" s="12"/>
-      <c r="F7" s="11" t="s">
-        <v>5</v>
+        <v>865</v>
+      </c>
+      <c r="D7" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B7,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E7" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B7,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B7,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F7" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B7,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>865</v>
+        <v>866</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>866</v>
+        <v>867</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>867</v>
-      </c>
-      <c r="D8" s="11"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="11" t="s">
-        <v>5</v>
+        <v>868</v>
+      </c>
+      <c r="D8" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B8,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E8" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B8,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B8,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F8" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B8,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>868</v>
+        <v>869</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>869</v>
+        <v>870</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>870</v>
-      </c>
-      <c r="D9" s="11"/>
-      <c r="E9" s="12"/>
-      <c r="F9" s="11" t="s">
-        <v>5</v>
+        <v>871</v>
+      </c>
+      <c r="D9" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B9,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E9" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B9,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B9,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F9" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B9,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>871</v>
+        <v>872</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>872</v>
+        <v>873</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>873</v>
-      </c>
-      <c r="D10" s="11"/>
-      <c r="E10" s="12"/>
-      <c r="F10" s="11" t="s">
-        <v>5</v>
+        <v>874</v>
+      </c>
+      <c r="D10" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B10,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E10" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B10,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B10,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B10,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>874</v>
+        <v>875</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>875</v>
+        <v>876</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>876</v>
-      </c>
-      <c r="D11" s="11"/>
-      <c r="E11" s="12"/>
-      <c r="F11" s="11" t="s">
-        <v>5</v>
+        <v>877</v>
+      </c>
+      <c r="D11" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B11,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E11" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B11,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B11,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B11,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>877</v>
+        <v>878</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>878</v>
+        <v>879</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>879</v>
-      </c>
-      <c r="D12" s="11"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="11" t="s">
-        <v>5</v>
+        <v>880</v>
+      </c>
+      <c r="D12" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B12,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E12" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B12,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B12,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B12,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>880</v>
+        <v>881</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>881</v>
+        <v>882</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>882</v>
-      </c>
-      <c r="D13" s="11"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="11" t="s">
-        <v>5</v>
+        <v>883</v>
+      </c>
+      <c r="D13" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$H$2:$H$204,MATCH(LEFT($B13,6),'Cas de test'!$A$2:$A$204,0))&amp;"","")</f>
+        <v/>
+      </c>
+      <c r="E13" s="13" t="str">
+        <f aca="false">IFERROR(IF(INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B13,6),'Cas de test'!$A$2:$A$204,0))="","",INDEX('Cas de test'!$I$2:$I$204,MATCH(LEFT($B13,6),'Cas de test'!$A$2:$A$204,0))),"")</f>
+        <v/>
+      </c>
+      <c r="F13" s="10" t="str">
+        <f aca="false">IFERROR(INDEX('Cas de test'!$J$2:$J$204,MATCH(LEFT($B13,6),'Cas de test'!$A$2:$A$204,0)),"Cas introuvable")</f>
+        <v>À faire</v>
       </c>
       <c r="G13" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="8" t="s">
-        <v>883</v>
+        <v>884</v>
       </c>
       <c r="C15" s="8" t="str">
         <f aca="false">COUNTIF(F2:F13,"OK")&amp;"/"&amp;COUNTA(B2:B13)</f>
         <v>0/12</v>
       </c>
     </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="8" t="s">
+        <v>885</v>
+      </c>
+      <c r="C16" s="8" t="str">
+        <f aca="false">IF(COUNTIF(F2:F13,"KO")&gt;0,"ÉCHEC — mise en service bloquée",IF(COUNTIF(F2:F13,"OK")=COUNTA(B2:B13),"Smoke test réussi",IF(COUNTIF(F2:F13,"À faire")=COUNTA(B2:B13),"Non démarré","En cours")))</f>
+        <v>Non démarré</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B18" s="2" t="s">
+        <v>886</v>
+      </c>
+    </row>
   </sheetData>
-  <dataValidations count="1">
-    <dataValidation allowBlank="false" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="F2:F13" type="list">
-      <formula1>"À faire,OK,KO,Bloqué"</formula1>
-      <formula2>0</formula2>
-    </dataValidation>
-  </dataValidations>
+  <conditionalFormatting sqref="F2:F13">
+    <cfRule type="cellIs" priority="2" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
+      <formula>"OK"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
+      <formula>"KO"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
+      <formula>"Bloqué"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="5" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
+      <formula>"N/A"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -11419,77 +11539,77 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
-        <v>884</v>
+      <c r="A1" s="14" t="s">
+        <v>887</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="14" t="s">
-        <v>885</v>
+      <c r="A2" s="15" t="s">
+        <v>888</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>886</v>
-      </c>
-      <c r="C3" s="15"/>
+        <v>889</v>
+      </c>
+      <c r="C3" s="16"/>
       <c r="D3" s="2" t="s">
-        <v>887</v>
+        <v>890</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>888</v>
+        <v>891</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>890</v>
+        <v>893</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>891</v>
+        <v>894</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>892</v>
+        <v>895</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>893</v>
+        <v>896</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>894</v>
+        <v>897</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>895</v>
+        <v>898</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>896</v>
+        <v>899</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>897</v>
+        <v>900</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>898</v>
+        <v>901</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>899</v>
+        <v>902</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>900</v>
+        <v>903</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>52</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>901</v>
+        <v>904</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>902</v>
+        <v>905</v>
       </c>
       <c r="G6" s="10" t="s">
         <v>57</v>
@@ -11501,30 +11621,30 @@
         <v>57</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>903</v>
+        <v>906</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>904</v>
+        <v>907</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>905</v>
+        <v>908</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>906</v>
+        <v>909</v>
       </c>
       <c r="D7" s="10" t="s">
         <v>52</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>907</v>
+        <v>910</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>908</v>
+        <v>911</v>
       </c>
       <c r="G7" s="10" t="s">
         <v>57</v>
@@ -11536,10 +11656,10 @@
         <v>57</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>909</v>
+        <v>912</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>910</v>
+        <v>913</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11550,124 +11670,124 @@
         <v>9001</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>911</v>
+        <v>914</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>66</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>913</v>
+        <v>916</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>915</v>
+        <v>918</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>916</v>
+        <v>919</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>917</v>
+        <v>920</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>918</v>
+        <v>921</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>920</v>
+        <v>923</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>66</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>921</v>
+        <v>924</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>922</v>
+        <v>925</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>923</v>
+        <v>926</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>924</v>
+        <v>927</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>925</v>
+        <v>928</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>926</v>
+        <v>929</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="B10" s="10" t="n">
         <v>9003</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>928</v>
+        <v>931</v>
       </c>
       <c r="D10" s="10" t="s">
         <v>66</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>929</v>
+        <v>932</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>930</v>
+        <v>933</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>850</v>
+        <v>851</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>931</v>
+        <v>934</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>932</v>
+        <v>935</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>933</v>
+        <v>936</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>934</v>
+        <v>937</v>
       </c>
       <c r="B11" s="10" t="n">
         <v>9004</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>935</v>
+        <v>938</v>
       </c>
       <c r="D11" s="10" t="s">
         <v>66</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>936</v>
+        <v>939</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H11" s="10" t="s">
         <v>57</v>
@@ -11676,105 +11796,105 @@
         <v>57</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>937</v>
+        <v>940</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>938</v>
+        <v>941</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>939</v>
+        <v>942</v>
       </c>
       <c r="B12" s="10" t="n">
         <v>9005</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>940</v>
+        <v>943</v>
       </c>
       <c r="D12" s="10" t="s">
         <v>66</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>941</v>
+        <v>944</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>942</v>
+        <v>945</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>853</v>
+        <v>854</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>943</v>
+        <v>946</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>944</v>
+        <v>947</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>945</v>
+        <v>948</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>946</v>
+        <v>949</v>
       </c>
       <c r="B13" s="10" t="n">
         <v>9006</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>947</v>
+        <v>950</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>66</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>912</v>
+        <v>915</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>948</v>
+        <v>951</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>949</v>
+        <v>952</v>
       </c>
       <c r="I13" s="10" t="s">
         <v>57</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>950</v>
+        <v>953</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>951</v>
+        <v>954</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
-        <v>952</v>
+        <v>955</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="s">
-        <v>953</v>
+      <c r="A16" s="15" t="s">
+        <v>956</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="s">
-        <v>954</v>
+      <c r="A17" s="15" t="s">
+        <v>957</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="14" t="s">
-        <v>955</v>
+      <c r="A18" s="15" t="s">
+        <v>958</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="14" t="s">
-        <v>956</v>
+      <c r="A19" s="15" t="s">
+        <v>959</v>
       </c>
     </row>
   </sheetData>
@@ -11806,56 +11926,56 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="13" t="s">
-        <v>957</v>
+      <c r="A1" s="14" t="s">
+        <v>960</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>958</v>
+        <v>961</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>888</v>
+        <v>891</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>46</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>891</v>
+        <v>894</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>960</v>
+        <v>963</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>961</v>
+        <v>964</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>47</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>962</v>
+        <v>965</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>963</v>
+        <v>966</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>964</v>
+        <v>967</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>2</v>
@@ -11864,27 +11984,27 @@
         <v>6</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>966</v>
+        <v>969</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>967</v>
+        <v>970</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>968</v>
+        <v>971</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>969</v>
+        <v>972</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>2</v>
@@ -11893,27 +12013,27 @@
         <v>4</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>971</v>
+        <v>974</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>972</v>
+        <v>975</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>9003</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>973</v>
+        <v>976</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>974</v>
+        <v>977</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>1</v>
@@ -11922,27 +12042,27 @@
         <v>2</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>975</v>
+        <v>978</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>976</v>
+        <v>979</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>977</v>
+        <v>980</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>9004</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>978</v>
+        <v>981</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>2</v>
@@ -11951,27 +12071,27 @@
         <v>6</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>979</v>
+        <v>982</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>980</v>
+        <v>983</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>9005</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>981</v>
+        <v>984</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>982</v>
+        <v>985</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>1</v>
@@ -11980,27 +12100,27 @@
         <v>5</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>983</v>
+        <v>986</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>984</v>
+        <v>987</v>
       </c>
       <c r="B10" s="10" t="n">
         <v>9006</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>985</v>
+        <v>988</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>986</v>
+        <v>989</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>1</v>
@@ -12009,27 +12129,27 @@
         <v>10</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>975</v>
+        <v>978</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>987</v>
+        <v>990</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>988</v>
+        <v>991</v>
       </c>
       <c r="B11" s="10" t="n">
         <v>9007</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>989</v>
+        <v>992</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>990</v>
+        <v>993</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>2</v>
@@ -12038,27 +12158,27 @@
         <v>6</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>922</v>
+        <v>925</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>991</v>
+        <v>994</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>992</v>
+        <v>995</v>
       </c>
       <c r="B12" s="10" t="n">
         <v>9008</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>993</v>
+        <v>996</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="E12" s="10" t="n">
         <v>2</v>
@@ -12067,27 +12187,27 @@
         <v>6</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>994</v>
+        <v>997</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>995</v>
+        <v>998</v>
       </c>
       <c r="B13" s="10" t="n">
         <v>9009</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>996</v>
+        <v>999</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>997</v>
+        <v>1000</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>3</v>
@@ -12096,27 +12216,27 @@
         <v>4</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>998</v>
+        <v>1001</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>999</v>
+        <v>1002</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>9010</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>1000</v>
+        <v>1003</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>2</v>
@@ -12125,27 +12245,27 @@
         <v>6</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>1001</v>
+        <v>1004</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>1002</v>
+        <v>1005</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>9011</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>1003</v>
+        <v>1006</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>965</v>
+        <v>968</v>
       </c>
       <c r="E15" s="10" t="n">
         <v>2</v>
@@ -12154,27 +12274,27 @@
         <v>3</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>975</v>
+        <v>978</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>1004</v>
+        <v>1007</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>1005</v>
+        <v>1008</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>9020</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>1006</v>
+        <v>1009</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>1007</v>
+        <v>1010</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>1</v>
@@ -12183,27 +12303,27 @@
         <v>4</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>1008</v>
+        <v>1011</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>1009</v>
+        <v>1012</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>9021</v>
       </c>
       <c r="C17" s="10" t="s">
+        <v>1013</v>
+      </c>
+      <c r="D17" s="10" t="s">
         <v>1010</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>1007</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>1</v>
@@ -12212,27 +12332,27 @@
         <v>4</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>1011</v>
+        <v>1014</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>1012</v>
+        <v>1015</v>
       </c>
       <c r="B18" s="10" t="n">
         <v>9023</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>1013</v>
+        <v>1016</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>1007</v>
+        <v>1010</v>
       </c>
       <c r="E18" s="10" t="n">
         <v>1</v>
@@ -12241,27 +12361,27 @@
         <v>4</v>
       </c>
       <c r="G18" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>1014</v>
+        <v>1017</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>1015</v>
+        <v>1018</v>
       </c>
       <c r="B19" s="10" t="n">
         <v>9024</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>1016</v>
+        <v>1019</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>1007</v>
+        <v>1010</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>1</v>
@@ -12270,157 +12390,157 @@
         <v>1</v>
       </c>
       <c r="G19" s="10" t="s">
-        <v>914</v>
+        <v>917</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>970</v>
+        <v>973</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>1017</v>
+        <v>1020</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>1018</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>1019</v>
+        <v>1022</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>1020</v>
+        <v>1023</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>1021</v>
+        <v>1024</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3" t="s">
-        <v>1022</v>
+        <v>1025</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>1023</v>
+        <v>1026</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>1024</v>
+        <v>1027</v>
       </c>
       <c r="B23" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>1025</v>
+        <v>1028</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>1026</v>
+        <v>1029</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
       <c r="G23" s="10"/>
       <c r="H23" s="10" t="s">
-        <v>1027</v>
+        <v>1030</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>1028</v>
+        <v>1031</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>1029</v>
+        <v>1032</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>1030</v>
+        <v>1033</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>1026</v>
+        <v>1029</v>
       </c>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10" t="s">
-        <v>1031</v>
+        <v>1034</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>1032</v>
+        <v>1035</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>1033</v>
+        <v>1036</v>
       </c>
       <c r="B25" s="10" t="n">
         <v>9003</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>1034</v>
+        <v>1037</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>1026</v>
+        <v>1029</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="10" t="s">
-        <v>1035</v>
+        <v>1038</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>1036</v>
+        <v>1039</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>1037</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>1038</v>
+        <v>1041</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>1020</v>
+        <v>1023</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>1039</v>
+        <v>1042</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>891</v>
+        <v>894</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>1040</v>
+        <v>1043</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>1041</v>
+        <v>1044</v>
       </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B29" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>1042</v>
+        <v>1045</v>
       </c>
       <c r="D29" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>1043</v>
+        <v>1046</v>
       </c>
       <c r="F29" s="10" t="n">
         <v>1</v>
@@ -12433,19 +12553,19 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>939</v>
+        <v>942</v>
       </c>
       <c r="B30" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>1042</v>
+        <v>1045</v>
       </c>
       <c r="D30" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>1044</v>
+        <v>1047</v>
       </c>
       <c r="F30" s="10" t="n">
         <v>1</v>
@@ -12464,13 +12584,13 @@
         <v>9003</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>1045</v>
+        <v>1048</v>
       </c>
       <c r="D31" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>1043</v>
+        <v>1046</v>
       </c>
       <c r="F31" s="10" t="n">
         <v>2</v>
@@ -12483,19 +12603,19 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B32" s="10" t="n">
         <v>9004</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>1045</v>
+        <v>1048</v>
       </c>
       <c r="D32" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>1046</v>
+        <v>1049</v>
       </c>
       <c r="F32" s="10" t="n">
         <v>4</v>
@@ -12508,19 +12628,19 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>939</v>
+        <v>942</v>
       </c>
       <c r="B33" s="10" t="n">
         <v>9005</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>1045</v>
+        <v>1048</v>
       </c>
       <c r="D33" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>1044</v>
+        <v>1047</v>
       </c>
       <c r="F33" s="10" t="n">
         <v>2</v>
@@ -12539,13 +12659,13 @@
         <v>9006</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>1047</v>
+        <v>1050</v>
       </c>
       <c r="D34" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>1043</v>
+        <v>1046</v>
       </c>
       <c r="F34" s="10" t="n">
         <v>3</v>
@@ -12558,19 +12678,19 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="10" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B35" s="10" t="n">
         <v>9007</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>1047</v>
+        <v>1050</v>
       </c>
       <c r="D35" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>1046</v>
+        <v>1049</v>
       </c>
       <c r="F35" s="10" t="n">
         <v>6</v>
@@ -12583,19 +12703,19 @@
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="10" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B36" s="10" t="n">
         <v>9008</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>1048</v>
+        <v>1051</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>1043</v>
+        <v>1046</v>
       </c>
       <c r="F36" s="10" t="n">
         <v>2</v>
@@ -12608,19 +12728,19 @@
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="10" t="s">
-        <v>939</v>
+        <v>942</v>
       </c>
       <c r="B37" s="10" t="n">
         <v>9009</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>1048</v>
+        <v>1051</v>
       </c>
       <c r="D37" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>1044</v>
+        <v>1047</v>
       </c>
       <c r="F37" s="10" t="n">
         <v>2</v>
@@ -12633,19 +12753,19 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="10" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B38" s="10" t="n">
         <v>9010</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>1049</v>
+        <v>1052</v>
       </c>
       <c r="D38" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>1043</v>
+        <v>1046</v>
       </c>
       <c r="F38" s="10" t="n">
         <v>1</v>
@@ -12664,13 +12784,13 @@
         <v>9011</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>1050</v>
+        <v>1053</v>
       </c>
       <c r="D39" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>1043</v>
+        <v>1046</v>
       </c>
       <c r="F39" s="10" t="n">
         <v>2</v>
@@ -12683,19 +12803,19 @@
     </row>
     <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="s">
-        <v>939</v>
+        <v>942</v>
       </c>
       <c r="B40" s="10" t="n">
         <v>9012</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>1051</v>
+        <v>1054</v>
       </c>
       <c r="D40" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>1044</v>
+        <v>1047</v>
       </c>
       <c r="F40" s="10" t="n">
         <v>1</v>
@@ -12708,39 +12828,39 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>1052</v>
+        <v>1055</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>1038</v>
+        <v>1041</v>
       </c>
       <c r="B43" s="3" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="C43" s="3" t="s">
         <v>46</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>959</v>
+        <v>962</v>
       </c>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3" t="s">
-        <v>1053</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="10" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B44" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>1054</v>
+        <v>1057</v>
       </c>
       <c r="D44" s="10" t="n">
         <v>3</v>
@@ -12750,18 +12870,18 @@
       <c r="G44" s="10"/>
       <c r="H44" s="10"/>
       <c r="I44" s="10" t="s">
-        <v>1055</v>
+        <v>1058</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="10" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="B45" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>1056</v>
+        <v>1059</v>
       </c>
       <c r="D45" s="10" t="n">
         <v>2</v>
@@ -12771,24 +12891,24 @@
       <c r="G45" s="10"/>
       <c r="H45" s="10"/>
       <c r="I45" s="10" t="s">
-        <v>1057</v>
+        <v>1060</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>1058</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>1038</v>
+        <v>1041</v>
       </c>
       <c r="B48" s="3"/>
       <c r="C48" s="3" t="s">
-        <v>1059</v>
+        <v>1062</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>1060</v>
+        <v>1063</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>29</v>
@@ -12820,7 +12940,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="10" t="s">
-        <v>919</v>
+        <v>922</v>
       </c>
       <c r="B50" s="10"/>
       <c r="C50" s="10" t="n">
@@ -12837,12 +12957,12 @@
       <c r="G50" s="10"/>
       <c r="H50" s="10"/>
       <c r="I50" s="10" t="s">
-        <v>1061</v>
+        <v>1064</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="10" t="s">
-        <v>927</v>
+        <v>930</v>
       </c>
       <c r="B51" s="10"/>
       <c r="C51" s="10" t="n">
@@ -12862,30 +12982,30 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="8" t="s">
-        <v>1062</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>1063</v>
+        <v>1066</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>1064</v>
+        <v>1067</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>1065</v>
+        <v>1068</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>1066</v>
+        <v>1069</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>1038</v>
+        <v>1041</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
       <c r="H54" s="3"/>
       <c r="I54" s="3" t="s">
-        <v>1067</v>
+        <v>1070</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12896,19 +13016,19 @@
         <v>9001</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>1068</v>
+        <v>1071</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>1069</v>
+        <v>1072</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>1070</v>
+        <v>1073</v>
       </c>
       <c r="F55" s="10"/>
       <c r="G55" s="10"/>
       <c r="H55" s="10"/>
       <c r="I55" s="10" t="s">
-        <v>1071</v>
+        <v>1074</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12919,19 +13039,19 @@
         <v>9001</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>1068</v>
+        <v>1071</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>1069</v>
+        <v>1072</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>1072</v>
+        <v>1075</v>
       </c>
       <c r="F56" s="10"/>
       <c r="G56" s="10"/>
       <c r="H56" s="10"/>
       <c r="I56" s="10" t="s">
-        <v>1073</v>
+        <v>1076</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12942,19 +13062,19 @@
         <v>9001</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>1068</v>
+        <v>1071</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>1069</v>
+        <v>1072</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>1074</v>
+        <v>1077</v>
       </c>
       <c r="F57" s="10"/>
       <c r="G57" s="10"/>
       <c r="H57" s="10"/>
       <c r="I57" s="10" t="s">
-        <v>1075</v>
+        <v>1078</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12965,19 +13085,19 @@
         <v>9002</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>1076</v>
+        <v>1079</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>1077</v>
+        <v>1080</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>1078</v>
+        <v>1081</v>
       </c>
       <c r="F58" s="10"/>
       <c r="G58" s="10"/>
       <c r="H58" s="10"/>
       <c r="I58" s="10" t="s">
-        <v>1079</v>
+        <v>1082</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12988,35 +13108,35 @@
         <v>9001</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>1068</v>
+        <v>1071</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>1080</v>
+        <v>1083</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>1078</v>
+        <v>1081</v>
       </c>
       <c r="F59" s="10"/>
       <c r="G59" s="10"/>
       <c r="H59" s="10"/>
       <c r="I59" s="10" t="s">
-        <v>1081</v>
+        <v>1084</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
-        <v>1082</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>1083</v>
+        <v>1086</v>
       </c>
       <c r="B62" s="3" t="s">
-        <v>889</v>
+        <v>892</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>1084</v>
+        <v>1087</v>
       </c>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
@@ -13033,7 +13153,7 @@
         <v>9001</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>1085</v>
+        <v>1088</v>
       </c>
       <c r="D63" s="10"/>
       <c r="E63" s="10"/>
@@ -13044,13 +13164,13 @@
     </row>
     <row r="64" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="10" t="s">
-        <v>1086</v>
+        <v>1089</v>
       </c>
       <c r="B64" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>1087</v>
+        <v>1090</v>
       </c>
       <c r="D64" s="10"/>
       <c r="E64" s="10"/>
@@ -13061,13 +13181,13 @@
     </row>
     <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="10" t="s">
-        <v>1088</v>
+        <v>1091</v>
       </c>
       <c r="B65" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>1089</v>
+        <v>1092</v>
       </c>
       <c r="D65" s="10"/>
       <c r="E65" s="10"/>
@@ -13078,13 +13198,13 @@
     </row>
     <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="10" t="s">
-        <v>1088</v>
+        <v>1091</v>
       </c>
       <c r="B66" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>1090</v>
+        <v>1093</v>
       </c>
       <c r="D66" s="10"/>
       <c r="E66" s="10"/>
@@ -13095,13 +13215,13 @@
     </row>
     <row r="67" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="10" t="s">
-        <v>1088</v>
+        <v>1091</v>
       </c>
       <c r="B67" s="10" t="n">
         <v>9003</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>1091</v>
+        <v>1094</v>
       </c>
       <c r="D67" s="10"/>
       <c r="E67" s="10"/>
@@ -13112,13 +13232,13 @@
     </row>
     <row r="68" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
-        <v>1092</v>
+        <v>1095</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>1093</v>
+        <v>1096</v>
       </c>
       <c r="D68" s="10"/>
       <c r="E68" s="10"/>
@@ -13154,13 +13274,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>1094</v>
+        <v>1097</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1095</v>
+        <v>1098</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1096</v>
+        <v>1099</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>49</v>
@@ -13168,397 +13288,397 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>1098</v>
+        <v>1101</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>1100</v>
+        <v>1103</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1101</v>
+        <v>1104</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B5" s="10" t="s">
+        <v>1105</v>
+      </c>
+      <c r="C5" s="11" t="s">
         <v>1102</v>
-      </c>
-      <c r="C5" s="11" t="s">
-        <v>1099</v>
       </c>
       <c r="D5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1103</v>
+        <v>1106</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D6" s="11"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>1104</v>
+        <v>1107</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>1105</v>
+        <v>1108</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1097</v>
+        <v>1100</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>1106</v>
+        <v>1109</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>1108</v>
+        <v>1111</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>1109</v>
+        <v>1112</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>1110</v>
+        <v>1113</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>1111</v>
+        <v>1114</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>1112</v>
+        <v>1115</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>1113</v>
+        <v>1116</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>1114</v>
+        <v>1117</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>1115</v>
+        <v>1118</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>1116</v>
+        <v>1119</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>1117</v>
+        <v>1120</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>1118</v>
+        <v>1121</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>1119</v>
+        <v>1122</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>1120</v>
+        <v>1123</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>1121</v>
+        <v>1124</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>1122</v>
+        <v>1125</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>1107</v>
+        <v>1110</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>1123</v>
+        <v>1126</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>1125</v>
+        <v>1128</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>1126</v>
+        <v>1129</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>1127</v>
+        <v>1130</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>1124</v>
+        <v>1127</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>1128</v>
+        <v>1131</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1130</v>
+        <v>1133</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>1131</v>
+        <v>1134</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>1132</v>
+        <v>1135</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>1133</v>
+        <v>1136</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>1129</v>
+        <v>1132</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>1134</v>
+        <v>1137</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>1099</v>
+        <v>1102</v>
       </c>
       <c r="D34" s="11"/>
     </row>
@@ -13605,25 +13725,25 @@
         <v>39</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1135</v>
+        <v>1138</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1136</v>
+        <v>1139</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>1137</v>
+        <v>1140</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>1138</v>
+        <v>1141</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>1139</v>
+        <v>1142</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>1140</v>
+        <v>1143</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>1141</v>
+        <v>1144</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>44</v>
@@ -13632,7 +13752,7 @@
         <v>47</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>1142</v>
+        <v>1145</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>46</v>
@@ -13640,34 +13760,34 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>1143</v>
+        <v>1146</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>181</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1144</v>
+        <v>1147</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>1145</v>
+        <v>1148</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>68</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>1146</v>
+        <v>1149</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>1147</v>
+        <v>1150</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>1148</v>
+        <v>1151</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>1149</v>
+        <v>1152</v>
       </c>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
@@ -14472,7 +14592,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>1150</v>
+        <v>1153</v>
       </c>
     </row>
   </sheetData>
@@ -14511,21 +14631,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>1151</v>
+        <v>1154</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1152</v>
+        <v>1155</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1153</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>1154</v>
+        <v>1157</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>1155</v>
+        <v>1158</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>169</v>
@@ -14533,65 +14653,65 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>1156</v>
+        <v>1159</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>1157</v>
+        <v>1160</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>1158</v>
+        <v>1161</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>1159</v>
+        <v>1162</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1160</v>
+        <v>1163</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>1161</v>
+        <v>1164</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>1162</v>
+        <v>1165</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>1163</v>
+        <v>1166</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>1164</v>
+        <v>1167</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>1165</v>
+        <v>1168</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1166</v>
+        <v>1169</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>1167</v>
+        <v>1170</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>1168</v>
+        <v>1171</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>1169</v>
+        <v>1172</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>1170</v>
+        <v>1173</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>1171</v>
+        <v>1174</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>1172</v>
+        <v>1175</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>450</v>
@@ -14599,10 +14719,10 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1173</v>
+        <v>1176</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>1174</v>
+        <v>1177</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>679</v>

</xml_diff>

<commit_message>
Cohérence plan de test / jeu de données / tests automatisés
- Plan (§ 15) aligné sur le jeu de test : comptes, sessions, jetons, CSV
- TRV-08 avant TRV-05 (U-FAM1 déjà inscrite), TRV-11 sur T-DERNIERE-PLACE,
  CRO-03 (3 mails) et CRO-06 (argument 10)
- Doc : 36 tests PHPUnit, CI GitHub Actions existante, couverture croisée
- Jeu SQL : purge des familles ZZIMPORT et des membres/e-mails ajoutés par
  import (rechargement rejouable) ; références de cas et chemins CI4 à jour
- Classeur régénéré

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Fg2rtdM1t4DnuUp3bsGB2V
</commit_message>
<xml_diff>
--- a/plan_tests_site_travaux.xlsx
+++ b/plan_tests_site_travaux.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2190" uniqueCount="1178">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2191" uniqueCount="1179">
   <si>
     <t xml:space="preserve">Plan de test — site_travaux (ABCM Mulhouse-Lutterbach)</t>
   </si>
@@ -557,7 +557,7 @@
     <t xml:space="preserve">Inscription</t>
   </si>
   <si>
-    <t xml:space="preserve">register_one/&lt;T-FUTUR&gt;, type_participant = Mr</t>
+    <t xml:space="preserve">En U-FAM1, après TRV-08 (le jeu l'inscrit déjà à T-FUTUR) : register_one/&lt;T-FUTUR&gt;, type_participant = Mr</t>
   </si>
   <si>
     <t xml:space="preserve">infos créé avec nb_participants=1, unités prévues = nb_units, redirection avec confirmation</t>
@@ -629,7 +629,7 @@
     <t xml:space="preserve">Concurrence sur la dernière place</t>
   </si>
   <si>
-    <t xml:space="preserve">Deux navigateurs, deux familles, dernière place de T-FUTUR, valider quasi simultanément</t>
+    <t xml:space="preserve">Deux navigateurs, deux familles non inscrites (U-FAM1 et U-REF), dernière place de T-DERNIERE-PLACE, valider quasi simultanément</t>
   </si>
   <si>
     <t xml:space="preserve">Une seule inscription acceptée ; l'autre reçoit TOO_MANY_PEOPLE (à défaut, ouvrir une anomalie sur le contrôle de capacité)</t>
@@ -1661,10 +1661,10 @@
     <t xml:space="preserve">Taille du lot</t>
   </si>
   <si>
-    <t xml:space="preserve">cron sendmail 2 avec 5 mails en attente</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Exactement 2 traités</t>
+    <t xml:space="preserve">cron sendmail 2 avec les 3 mails du jeu en attente (recharger le jeu après CRO-01)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exactement 2 traités, 1 reste en statut=0</t>
   </si>
   <si>
     <t xml:space="preserve">CRO-04</t>
@@ -1697,10 +1697,10 @@
     <t xml:space="preserve">Mails de validation référent</t>
   </si>
   <si>
-    <t xml:space="preserve">php spark cron:ref-validation 7 avec une session à J+5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Token créé (expiration J+30), mail poussé en file, travaux.ref_mail_sent_at renseigné</t>
+    <t xml:space="preserve">php spark cron:ref-validation 10 (sessions MEN/TRA de J à J+10 avec référent : T-DERNIERE-PLACE J+8, T-PLEIN J+10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 tokens créés (expiration J+30), 2 mails poussés en file, travaux.ref_mail_sent_at renseigné ; avec l'argument 7 par défaut, seule T-REF-KO (J+6) est candidate (voir CRO-08)</t>
   </si>
   <si>
     <t xml:space="preserve">CRO-07</t>
@@ -1721,7 +1721,7 @@
     <t xml:space="preserve">Référent introuvable</t>
   </si>
   <si>
-    <t xml:space="preserve">Session sans référent ou chaîne trombi cassée</t>
+    <t xml:space="preserve">Session sans référent ou chaîne trombi cassée (T-REF-KO)</t>
   </si>
   <si>
     <t xml:space="preserve">Session ignorée sans erreur, trace en log</t>
@@ -2606,21 +2606,21 @@
     <t xml:space="preserve">4</t>
   </si>
   <si>
+    <t xml:space="preserve">TRV-08 — Désinscription (U-FAM1 est déjà inscrite à T-FUTUR)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ligne supprimée, place libérée</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5</t>
+  </si>
+  <si>
     <t xml:space="preserve">TRV-05 — Inscription à une session</t>
   </si>
   <si>
     <t xml:space="preserve">Ligne créée dans infos, compteur d'inscrits incrémenté</t>
   </si>
   <si>
-    <t xml:space="preserve">5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TRV-08 — Désinscription</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ligne supprimée, place libérée</t>
-  </si>
-  <si>
     <t xml:space="preserve">6</t>
   </si>
   <si>
@@ -2795,7 +2795,7 @@
     <t xml:space="preserve">Parcours nominal, 0 unité validée. Inscrite à T-FUTUR (désinscription) et à T-PASSE, T-ACTION. 2 e-mails complémentaires (conjoint, contact de secours). Second référent de session (trombi 9003).</t>
   </si>
   <si>
-    <t xml:space="preserve">AUT-04, TRV-01 à TRV-10, FAM-01, FAM-04, CAN-*, ACL-11, MAI-01</t>
+    <t xml:space="preserve">AUT-04, TRV-01 à TRV-10 (TRV-08 avant TRV-05), TRV-11, FAM-01, FAM-04, CAN-*, ACL-11, MAI-01</t>
   </si>
   <si>
     <t xml:space="preserve">U-FAM2</t>
@@ -2840,7 +2840,7 @@
     <t xml:space="preserve">Référente principale (trombi 9001, classif reftra) de T-FUTUR, T-PASSE, T-ACTION, T-VIEUX… 2 unités complémentaires. Porte les 3 jetons de validation.</t>
   </si>
   <si>
-    <t xml:space="preserve">REF-01 à REF-11, MAI-01, CRO-06, CRO-07</t>
+    <t xml:space="preserve">REF-01 à REF-11, MAI-01, CRO-06 (argument 10), CRO-07</t>
   </si>
   <si>
     <t xml:space="preserve">U-LEGACY</t>
@@ -2876,7 +2876,7 @@
     <t xml:space="preserve">Inscrite à T-PLEIN, T-PASSE, T-DERNIERE-PLACE et au créneau cantine du vendredi (saturé). Responsable de commission BUREAU (trombi RT) et membre simple TRAVAUX (ME).</t>
   </si>
   <si>
-    <t xml:space="preserve">CAN-05, TRV-07, TRV-11, ORG-01</t>
+    <t xml:space="preserve">CAN-05, TRV-07, ORG-01</t>
   </si>
   <si>
     <t xml:space="preserve">U-FAM4</t>
@@ -2897,13 +2897,16 @@
     <t xml:space="preserve">IMP-01 à IMP-09</t>
   </si>
   <si>
-    <t xml:space="preserve">Écarts avec le § 15.4.1 de DOCUMENTATION.md</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• Les logins du plan (admin, gestion@test.local, famille1@test.local…) sont remplacés par ceux du jeu de test : admin.recette@, restreint.recette@, famille1@… (domaine @recette.local, modifiable via @MAIL_DOM dans le script SQL).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">• U-FAM3 (école B) et U-FAM4 (cible d'import) n'existent que dans le jeu de test ; U-DELTA (SSO) n'est pas créé par le jeu : prévoir un compte Delta réel pour AUT-06.</t>
+    <t xml:space="preserve">Remarques</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• Le plan (§ 15.4 de DOCUMENTATION.md) est aligné sur ce jeu de test : mêmes logins, mêmes sessions, mêmes jetons.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• U-DELTA (SSO, AUT-06) n'est pas créé par le jeu : prévoir un compte Delta réel.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">• U-FAM1 est déjà inscrite à T-FUTUR : exécuter TRV-08 (désinscription) avant TRV-05 (inscription), comme dans le smoke test.</t>
   </si>
   <si>
     <t xml:space="preserve">• Tous les identifiants du jeu sont dans la plage 9000–9999 ; retrait complet avec 90_purge_jeu_de_test.sql ou POST Api/jeu_de_test {"action":"purge"} (travaux.allowTestData requis).</t>
@@ -3053,7 +3056,7 @@
     <t xml:space="preserve">J+8</t>
   </si>
   <si>
-    <t xml:space="preserve">2 places prises sur 3 ; second référent (Martin Claire) : concurrence (TRV-11, PER-04)</t>
+    <t xml:space="preserve">2 places prises sur 3 (U-FAM2, U-FAM3) ; second référent (Martin Claire) : concurrence avec U-FAM1 et U-REF (TRV-11, PER-04) ; candidate de CRO-06</t>
   </si>
   <si>
     <t xml:space="preserve">T-CAN lundi</t>
@@ -3353,7 +3356,7 @@
     <t xml:space="preserve">Droits d'écriture sur writable/, public/files/, app/Language/.</t>
   </si>
   <si>
-    <t xml:space="preserve">travaux.civilYear (.env) cohérent avec les données de test (par défaut 2025-2026).</t>
+    <t xml:space="preserve">travaux.civilYear (.env) cohérent avec les données de test (par défaut 2025-2026 ; adapter à la campagne en cours — Api/jeu_de_test reprend cette valeur).</t>
   </si>
   <si>
     <t xml:space="preserve">travaux.maintenance = false, travaux.debugApp = none (sauf test dédié) et CI_ENVIRONMENT = production.</t>
@@ -8681,7 +8684,7 @@
       <c r="K122" s="11"/>
       <c r="L122" s="11"/>
     </row>
-    <row r="123" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="10" t="s">
         <v>541</v>
       </c>
@@ -8771,7 +8774,7 @@
       <c r="K125" s="11"/>
       <c r="L125" s="11"/>
     </row>
-    <row r="126" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="126" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A126" s="10" t="s">
         <v>553</v>
       </c>
@@ -11254,7 +11257,7 @@
       </c>
       <c r="G4" s="11"/>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
         <v>857</v>
       </c>
@@ -11523,7 +11526,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K19"/>
+  <dimension ref="A1:K20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -11895,6 +11898,11 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="15" t="s">
         <v>959</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="15" t="s">
+        <v>960</v>
       </c>
     </row>
   </sheetData>
@@ -11927,12 +11935,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="14" t="s">
-        <v>960</v>
+        <v>961</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
-        <v>961</v>
+        <v>962</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -11949,33 +11957,33 @@
         <v>894</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>963</v>
+        <v>964</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>964</v>
+        <v>965</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>47</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>965</v>
+        <v>966</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>966</v>
+        <v>967</v>
       </c>
       <c r="B5" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>967</v>
+        <v>968</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>2</v>
@@ -11987,24 +11995,24 @@
         <v>917</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>969</v>
+        <v>970</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>970</v>
+        <v>971</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>971</v>
+        <v>972</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>972</v>
+        <v>973</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>2</v>
@@ -12016,24 +12024,24 @@
         <v>917</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>974</v>
+        <v>975</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>975</v>
+        <v>976</v>
       </c>
       <c r="B7" s="10" t="n">
         <v>9003</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>976</v>
+        <v>977</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>977</v>
+        <v>978</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>1</v>
@@ -12042,27 +12050,27 @@
         <v>2</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>979</v>
+        <v>980</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>980</v>
+        <v>981</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>9004</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>981</v>
+        <v>982</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>2</v>
@@ -12074,24 +12082,24 @@
         <v>917</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>982</v>
+        <v>983</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>983</v>
+        <v>984</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>9005</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>984</v>
+        <v>985</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>985</v>
+        <v>986</v>
       </c>
       <c r="E9" s="10" t="n">
         <v>1</v>
@@ -12103,24 +12111,24 @@
         <v>917</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>986</v>
+        <v>987</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>987</v>
+        <v>988</v>
       </c>
       <c r="B10" s="10" t="n">
         <v>9006</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>988</v>
+        <v>989</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>989</v>
+        <v>990</v>
       </c>
       <c r="E10" s="10" t="n">
         <v>1</v>
@@ -12129,27 +12137,27 @@
         <v>10</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>990</v>
+        <v>991</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>991</v>
+        <v>992</v>
       </c>
       <c r="B11" s="10" t="n">
         <v>9007</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>992</v>
+        <v>993</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="E11" s="10" t="n">
         <v>2</v>
@@ -12161,24 +12169,24 @@
         <v>925</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>994</v>
+        <v>995</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>995</v>
+        <v>996</v>
       </c>
       <c r="B12" s="10" t="n">
         <v>9008</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>996</v>
+        <v>997</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="E12" s="10" t="n">
         <v>2</v>
@@ -12190,24 +12198,24 @@
         <v>917</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>997</v>
+        <v>998</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>998</v>
+        <v>999</v>
       </c>
       <c r="B13" s="10" t="n">
         <v>9009</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>999</v>
+        <v>1000</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>1000</v>
+        <v>1001</v>
       </c>
       <c r="E13" s="10" t="n">
         <v>3</v>
@@ -12219,24 +12227,24 @@
         <v>917</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>1001</v>
+        <v>1002</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>1002</v>
+        <v>1003</v>
       </c>
       <c r="B14" s="10" t="n">
         <v>9010</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>1003</v>
+        <v>1004</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="E14" s="10" t="n">
         <v>2</v>
@@ -12248,24 +12256,24 @@
         <v>917</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>1004</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>1005</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>1005</v>
+        <v>1006</v>
       </c>
       <c r="B15" s="10" t="n">
         <v>9011</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>1006</v>
+        <v>1007</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>968</v>
+        <v>969</v>
       </c>
       <c r="E15" s="10" t="n">
         <v>2</v>
@@ -12274,27 +12282,27 @@
         <v>3</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>978</v>
+        <v>979</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>1007</v>
+        <v>1008</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>1008</v>
+        <v>1009</v>
       </c>
       <c r="B16" s="10" t="n">
         <v>9020</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>1009</v>
+        <v>1010</v>
       </c>
       <c r="D16" s="10" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="E16" s="10" t="n">
         <v>1</v>
@@ -12306,24 +12314,24 @@
         <v>917</v>
       </c>
       <c r="H16" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I16" s="10" t="s">
-        <v>1011</v>
+        <v>1012</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>1012</v>
+        <v>1013</v>
       </c>
       <c r="B17" s="10" t="n">
         <v>9021</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>1013</v>
+        <v>1014</v>
       </c>
       <c r="D17" s="10" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="E17" s="10" t="n">
         <v>1</v>
@@ -12335,24 +12343,24 @@
         <v>917</v>
       </c>
       <c r="H17" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I17" s="10" t="s">
-        <v>1014</v>
+        <v>1015</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>1015</v>
+        <v>1016</v>
       </c>
       <c r="B18" s="10" t="n">
         <v>9023</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>1016</v>
+        <v>1017</v>
       </c>
       <c r="D18" s="10" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="E18" s="10" t="n">
         <v>1</v>
@@ -12364,24 +12372,24 @@
         <v>917</v>
       </c>
       <c r="H18" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I18" s="10" t="s">
-        <v>1017</v>
+        <v>1018</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>1018</v>
+        <v>1019</v>
       </c>
       <c r="B19" s="10" t="n">
         <v>9024</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>1019</v>
+        <v>1020</v>
       </c>
       <c r="D19" s="10" t="s">
-        <v>1010</v>
+        <v>1011</v>
       </c>
       <c r="E19" s="10" t="n">
         <v>1</v>
@@ -12393,135 +12401,135 @@
         <v>917</v>
       </c>
       <c r="H19" s="10" t="s">
-        <v>973</v>
+        <v>974</v>
       </c>
       <c r="I19" s="10" t="s">
-        <v>1020</v>
+        <v>1021</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="8" t="s">
-        <v>1021</v>
+        <v>1022</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>1022</v>
+        <v>1023</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>892</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>1024</v>
+        <v>1025</v>
       </c>
       <c r="E22" s="3"/>
       <c r="F22" s="3"/>
       <c r="G22" s="3"/>
       <c r="H22" s="3" t="s">
-        <v>1025</v>
+        <v>1026</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>1026</v>
+        <v>1027</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>1027</v>
+        <v>1028</v>
       </c>
       <c r="B23" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>1028</v>
+        <v>1029</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="10"/>
       <c r="G23" s="10"/>
       <c r="H23" s="10" t="s">
-        <v>1030</v>
+        <v>1031</v>
       </c>
       <c r="I23" s="10" t="s">
-        <v>1031</v>
+        <v>1032</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>1032</v>
+        <v>1033</v>
       </c>
       <c r="B24" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>1033</v>
+        <v>1034</v>
       </c>
       <c r="D24" s="10" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="E24" s="10"/>
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10" t="s">
-        <v>1034</v>
+        <v>1035</v>
       </c>
       <c r="I24" s="10" t="s">
-        <v>1035</v>
+        <v>1036</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>1036</v>
+        <v>1037</v>
       </c>
       <c r="B25" s="10" t="n">
         <v>9003</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>1037</v>
+        <v>1038</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>1029</v>
+        <v>1030</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="10" t="s">
-        <v>1038</v>
+        <v>1039</v>
       </c>
       <c r="I25" s="10" t="s">
-        <v>1039</v>
+        <v>1040</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="8" t="s">
-        <v>1040</v>
+        <v>1041</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>892</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>1023</v>
+        <v>1024</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>1042</v>
+        <v>1043</v>
       </c>
       <c r="E28" s="3" t="s">
         <v>894</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>1043</v>
+        <v>1044</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>1044</v>
+        <v>1045</v>
       </c>
       <c r="H28" s="3"/>
       <c r="I28" s="3"/>
@@ -12534,13 +12542,13 @@
         <v>9001</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="D29" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F29" s="10" t="n">
         <v>1</v>
@@ -12559,13 +12567,13 @@
         <v>9002</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>1045</v>
+        <v>1046</v>
       </c>
       <c r="D30" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="F30" s="10" t="n">
         <v>1</v>
@@ -12584,13 +12592,13 @@
         <v>9003</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="D31" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F31" s="10" t="n">
         <v>2</v>
@@ -12609,13 +12617,13 @@
         <v>9004</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="D32" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E32" s="10" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="F32" s="10" t="n">
         <v>4</v>
@@ -12634,13 +12642,13 @@
         <v>9005</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>1048</v>
+        <v>1049</v>
       </c>
       <c r="D33" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="F33" s="10" t="n">
         <v>2</v>
@@ -12659,13 +12667,13 @@
         <v>9006</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="D34" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E34" s="10" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F34" s="10" t="n">
         <v>3</v>
@@ -12684,13 +12692,13 @@
         <v>9007</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>1050</v>
+        <v>1051</v>
       </c>
       <c r="D35" s="10" t="n">
         <v>2</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>1049</v>
+        <v>1050</v>
       </c>
       <c r="F35" s="10" t="n">
         <v>6</v>
@@ -12709,13 +12717,13 @@
         <v>9008</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="D36" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E36" s="10" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F36" s="10" t="n">
         <v>2</v>
@@ -12734,13 +12742,13 @@
         <v>9009</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>1051</v>
+        <v>1052</v>
       </c>
       <c r="D37" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="F37" s="10" t="n">
         <v>2</v>
@@ -12759,13 +12767,13 @@
         <v>9010</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>1052</v>
+        <v>1053</v>
       </c>
       <c r="D38" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E38" s="10" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F38" s="10" t="n">
         <v>1</v>
@@ -12784,13 +12792,13 @@
         <v>9011</v>
       </c>
       <c r="C39" s="10" t="s">
-        <v>1053</v>
+        <v>1054</v>
       </c>
       <c r="D39" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>1046</v>
+        <v>1047</v>
       </c>
       <c r="F39" s="10" t="n">
         <v>2</v>
@@ -12809,13 +12817,13 @@
         <v>9012</v>
       </c>
       <c r="C40" s="10" t="s">
-        <v>1054</v>
+        <v>1055</v>
       </c>
       <c r="D40" s="10" t="n">
         <v>1</v>
       </c>
       <c r="E40" s="10" t="s">
-        <v>1047</v>
+        <v>1048</v>
       </c>
       <c r="F40" s="10" t="n">
         <v>1</v>
@@ -12828,12 +12836,12 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="8" t="s">
-        <v>1055</v>
+        <v>1056</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="3" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>892</v>
@@ -12842,14 +12850,14 @@
         <v>46</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>962</v>
+        <v>963</v>
       </c>
       <c r="E43" s="3"/>
       <c r="F43" s="3"/>
       <c r="G43" s="3"/>
       <c r="H43" s="3"/>
       <c r="I43" s="3" t="s">
-        <v>1056</v>
+        <v>1057</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12860,7 +12868,7 @@
         <v>9001</v>
       </c>
       <c r="C44" s="10" t="s">
-        <v>1057</v>
+        <v>1058</v>
       </c>
       <c r="D44" s="10" t="n">
         <v>3</v>
@@ -12870,7 +12878,7 @@
       <c r="G44" s="10"/>
       <c r="H44" s="10"/>
       <c r="I44" s="10" t="s">
-        <v>1058</v>
+        <v>1059</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12881,7 +12889,7 @@
         <v>9002</v>
       </c>
       <c r="C45" s="10" t="s">
-        <v>1059</v>
+        <v>1060</v>
       </c>
       <c r="D45" s="10" t="n">
         <v>2</v>
@@ -12891,24 +12899,24 @@
       <c r="G45" s="10"/>
       <c r="H45" s="10"/>
       <c r="I45" s="10" t="s">
-        <v>1060</v>
+        <v>1061</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="8" t="s">
-        <v>1061</v>
+        <v>1062</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="B48" s="3"/>
       <c r="C48" s="3" t="s">
-        <v>1062</v>
+        <v>1063</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>1063</v>
+        <v>1064</v>
       </c>
       <c r="E48" s="3" t="s">
         <v>29</v>
@@ -12957,7 +12965,7 @@
       <c r="G50" s="10"/>
       <c r="H50" s="10"/>
       <c r="I50" s="10" t="s">
-        <v>1064</v>
+        <v>1065</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12982,30 +12990,30 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="8" t="s">
-        <v>1065</v>
+        <v>1066</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="B54" s="3" t="s">
-        <v>1067</v>
+        <v>1068</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>1068</v>
+        <v>1069</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>1069</v>
+        <v>1070</v>
       </c>
       <c r="E54" s="3" t="s">
-        <v>1041</v>
+        <v>1042</v>
       </c>
       <c r="F54" s="3"/>
       <c r="G54" s="3"/>
       <c r="H54" s="3"/>
       <c r="I54" s="3" t="s">
-        <v>1070</v>
+        <v>1071</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13016,19 +13024,19 @@
         <v>9001</v>
       </c>
       <c r="C55" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="D55" s="10" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>1073</v>
+        <v>1074</v>
       </c>
       <c r="F55" s="10"/>
       <c r="G55" s="10"/>
       <c r="H55" s="10"/>
       <c r="I55" s="10" t="s">
-        <v>1074</v>
+        <v>1075</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13039,19 +13047,19 @@
         <v>9001</v>
       </c>
       <c r="C56" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="D56" s="10" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="E56" s="10" t="s">
-        <v>1075</v>
+        <v>1076</v>
       </c>
       <c r="F56" s="10"/>
       <c r="G56" s="10"/>
       <c r="H56" s="10"/>
       <c r="I56" s="10" t="s">
-        <v>1076</v>
+        <v>1077</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13062,19 +13070,19 @@
         <v>9001</v>
       </c>
       <c r="C57" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="D57" s="10" t="s">
-        <v>1072</v>
+        <v>1073</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>1077</v>
+        <v>1078</v>
       </c>
       <c r="F57" s="10"/>
       <c r="G57" s="10"/>
       <c r="H57" s="10"/>
       <c r="I57" s="10" t="s">
-        <v>1078</v>
+        <v>1079</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13085,19 +13093,19 @@
         <v>9002</v>
       </c>
       <c r="C58" s="10" t="s">
-        <v>1079</v>
+        <v>1080</v>
       </c>
       <c r="D58" s="10" t="s">
-        <v>1080</v>
+        <v>1081</v>
       </c>
       <c r="E58" s="10" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="F58" s="10"/>
       <c r="G58" s="10"/>
       <c r="H58" s="10"/>
       <c r="I58" s="10" t="s">
-        <v>1082</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13108,35 +13116,35 @@
         <v>9001</v>
       </c>
       <c r="C59" s="10" t="s">
-        <v>1071</v>
+        <v>1072</v>
       </c>
       <c r="D59" s="10" t="s">
-        <v>1083</v>
+        <v>1084</v>
       </c>
       <c r="E59" s="10" t="s">
-        <v>1081</v>
+        <v>1082</v>
       </c>
       <c r="F59" s="10"/>
       <c r="G59" s="10"/>
       <c r="H59" s="10"/>
       <c r="I59" s="10" t="s">
-        <v>1084</v>
+        <v>1085</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="8" t="s">
-        <v>1085</v>
+        <v>1086</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>1086</v>
+        <v>1087</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>892</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>1087</v>
+        <v>1088</v>
       </c>
       <c r="D62" s="3"/>
       <c r="E62" s="3"/>
@@ -13153,7 +13161,7 @@
         <v>9001</v>
       </c>
       <c r="C63" s="10" t="s">
-        <v>1088</v>
+        <v>1089</v>
       </c>
       <c r="D63" s="10"/>
       <c r="E63" s="10"/>
@@ -13164,13 +13172,13 @@
     </row>
     <row r="64" customFormat="false" ht="113.4" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="10" t="s">
-        <v>1089</v>
+        <v>1090</v>
       </c>
       <c r="B64" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C64" s="10" t="s">
-        <v>1090</v>
+        <v>1091</v>
       </c>
       <c r="D64" s="10"/>
       <c r="E64" s="10"/>
@@ -13181,13 +13189,13 @@
     </row>
     <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="10" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="B65" s="10" t="n">
         <v>9001</v>
       </c>
       <c r="C65" s="10" t="s">
-        <v>1092</v>
+        <v>1093</v>
       </c>
       <c r="D65" s="10"/>
       <c r="E65" s="10"/>
@@ -13198,13 +13206,13 @@
     </row>
     <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="10" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="B66" s="10" t="n">
         <v>9002</v>
       </c>
       <c r="C66" s="10" t="s">
-        <v>1093</v>
+        <v>1094</v>
       </c>
       <c r="D66" s="10"/>
       <c r="E66" s="10"/>
@@ -13215,13 +13223,13 @@
     </row>
     <row r="67" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="10" t="s">
-        <v>1091</v>
+        <v>1092</v>
       </c>
       <c r="B67" s="10" t="n">
         <v>9003</v>
       </c>
       <c r="C67" s="10" t="s">
-        <v>1094</v>
+        <v>1095</v>
       </c>
       <c r="D67" s="10"/>
       <c r="E67" s="10"/>
@@ -13232,13 +13240,13 @@
     </row>
     <row r="68" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="10" t="s">
-        <v>1095</v>
+        <v>1096</v>
       </c>
       <c r="B68" s="10" t="s">
         <v>57</v>
       </c>
       <c r="C68" s="10" t="s">
-        <v>1096</v>
+        <v>1097</v>
       </c>
       <c r="D68" s="10"/>
       <c r="E68" s="10"/>
@@ -13274,13 +13282,13 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>1097</v>
+        <v>1098</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1098</v>
+        <v>1099</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1099</v>
+        <v>1100</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>49</v>
@@ -13288,397 +13296,397 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>1101</v>
+        <v>1102</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D2" s="11"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>1104</v>
+      </c>
+      <c r="C3" s="11" t="s">
         <v>1103</v>
-      </c>
-      <c r="C3" s="11" t="s">
-        <v>1102</v>
       </c>
       <c r="D3" s="11"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1104</v>
+        <v>1105</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D4" s="11"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>1105</v>
+        <v>1106</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D5" s="11"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1106</v>
+        <v>1107</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D6" s="11"/>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>1107</v>
+        <v>1108</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D7" s="11"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>1108</v>
+        <v>1109</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D8" s="11"/>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1100</v>
+        <v>1101</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>1109</v>
+        <v>1110</v>
       </c>
       <c r="C9" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D9" s="11"/>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>1111</v>
+        <v>1112</v>
       </c>
       <c r="C10" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D10" s="11"/>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>1112</v>
+        <v>1113</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>1113</v>
+        <v>1114</v>
       </c>
       <c r="C12" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D12" s="11"/>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>1114</v>
+        <v>1115</v>
       </c>
       <c r="C13" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D13" s="11"/>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>1115</v>
+        <v>1116</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D14" s="11"/>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>1116</v>
+        <v>1117</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D15" s="11"/>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>1117</v>
+        <v>1118</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>1118</v>
+        <v>1119</v>
       </c>
       <c r="C17" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D17" s="11"/>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>1119</v>
+        <v>1120</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D18" s="11"/>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B19" s="10" t="s">
-        <v>1120</v>
+        <v>1121</v>
       </c>
       <c r="C19" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D19" s="11"/>
     </row>
     <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B20" s="10" t="s">
-        <v>1121</v>
+        <v>1122</v>
       </c>
       <c r="C20" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D20" s="11"/>
     </row>
     <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B21" s="10" t="s">
-        <v>1122</v>
+        <v>1123</v>
       </c>
       <c r="C21" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D21" s="11"/>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B22" s="10" t="s">
-        <v>1123</v>
+        <v>1124</v>
       </c>
       <c r="C22" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D22" s="11"/>
     </row>
     <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B23" s="10" t="s">
-        <v>1124</v>
+        <v>1125</v>
       </c>
       <c r="C23" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B24" s="10" t="s">
-        <v>1125</v>
+        <v>1126</v>
       </c>
       <c r="C24" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D24" s="11"/>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="s">
-        <v>1110</v>
+        <v>1111</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>1126</v>
+        <v>1127</v>
       </c>
       <c r="C25" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D25" s="11"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="10" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B26" s="10" t="s">
-        <v>1128</v>
+        <v>1129</v>
       </c>
       <c r="C26" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D26" s="11"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B27" s="10" t="s">
-        <v>1129</v>
+        <v>1130</v>
       </c>
       <c r="C27" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D27" s="11"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>1130</v>
+        <v>1131</v>
       </c>
       <c r="C28" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D28" s="11"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="s">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>1131</v>
+        <v>1132</v>
       </c>
       <c r="C29" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D29" s="11"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="10" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>1133</v>
+        <v>1134</v>
       </c>
       <c r="C30" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D30" s="11"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="10" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>1134</v>
+        <v>1135</v>
       </c>
       <c r="C31" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D31" s="11"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="10" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>1135</v>
+        <v>1136</v>
       </c>
       <c r="C32" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D32" s="11"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>1136</v>
+        <v>1137</v>
       </c>
       <c r="C33" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="10" t="s">
-        <v>1132</v>
+        <v>1133</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>1137</v>
+        <v>1138</v>
       </c>
       <c r="C34" s="11" t="s">
-        <v>1102</v>
+        <v>1103</v>
       </c>
       <c r="D34" s="11"/>
     </row>
@@ -13725,25 +13733,25 @@
         <v>39</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1138</v>
+        <v>1139</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1139</v>
+        <v>1140</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>1140</v>
+        <v>1141</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>1141</v>
+        <v>1142</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>1142</v>
+        <v>1143</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>1143</v>
+        <v>1144</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>1144</v>
+        <v>1145</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>44</v>
@@ -13752,7 +13760,7 @@
         <v>47</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>1145</v>
+        <v>1146</v>
       </c>
       <c r="L1" s="3" t="s">
         <v>46</v>
@@ -13760,34 +13768,34 @@
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>1146</v>
+        <v>1147</v>
       </c>
       <c r="B2" s="11" t="s">
         <v>181</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>1147</v>
+        <v>1148</v>
       </c>
       <c r="D2" s="11" t="s">
-        <v>1148</v>
+        <v>1149</v>
       </c>
       <c r="E2" s="11" t="s">
         <v>68</v>
       </c>
       <c r="F2" s="11" t="s">
-        <v>1149</v>
+        <v>1150</v>
       </c>
       <c r="G2" s="11" t="s">
-        <v>1150</v>
+        <v>1151</v>
       </c>
       <c r="H2" s="11" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="I2" s="11" t="s">
-        <v>1151</v>
+        <v>1152</v>
       </c>
       <c r="J2" s="11" t="s">
-        <v>1152</v>
+        <v>1153</v>
       </c>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
@@ -14592,7 +14600,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="2" t="s">
-        <v>1153</v>
+        <v>1154</v>
       </c>
     </row>
   </sheetData>
@@ -14631,21 +14639,21 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>1154</v>
+        <v>1155</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>1155</v>
+        <v>1156</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>1156</v>
+        <v>1157</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="10" t="s">
-        <v>1157</v>
+        <v>1158</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>1158</v>
+        <v>1159</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>169</v>
@@ -14653,65 +14661,65 @@
     </row>
     <row r="3" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="10" t="s">
-        <v>1159</v>
+        <v>1160</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="10" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="10" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="10" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="10" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>450</v>
@@ -14719,10 +14727,10 @@
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="10" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>679</v>

</xml_diff>